<commit_message>
bug fix and new station added for testing
bug: sections with more than one switch interfacing with more than one NDZ would crash the program
</commit_message>
<xml_diff>
--- a/stations/output/CIS_Interlocking_Program.xlsx
+++ b/stations/output/CIS_Interlocking_Program.xlsx
@@ -462,15 +462,6 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right style="thin">
         <color theme="1"/>
@@ -479,37 +470,6 @@
         <color theme="1"/>
       </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -531,30 +491,6 @@
       <top style="thin">
         <color theme="1"/>
       </top>
-      <bottom style="thin">
-        <color theme="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color theme="1"/>
-      </left>
-      <right style="thin">
-        <color theme="1"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color theme="1"/>
       </bottom>
@@ -585,6 +521,39 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right style="thin">
         <color theme="1"/>
@@ -592,6 +561,15 @@
       <top style="medium">
         <color theme="1"/>
       </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
+      <top/>
       <bottom/>
       <diagonal/>
     </border>
@@ -609,6 +587,17 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="1"/>
+      </right>
       <top/>
       <bottom style="thin">
         <color theme="1"/>
@@ -639,12 +628,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color theme="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="84">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -788,9 +788,6 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="8" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -818,29 +815,42 @@
     <xf numFmtId="0" fontId="6" fillId="8" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="38" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="42" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1183,49 +1193,49 @@
       <c r="B1" s="21" t="n"/>
       <c r="C1" s="21" t="n"/>
       <c r="D1" s="21" t="n"/>
-      <c r="E1" s="59" t="inlineStr">
+      <c r="E1" s="61" t="inlineStr">
         <is>
           <t>ZIRCON</t>
         </is>
       </c>
-      <c r="F1" s="60" t="n"/>
+      <c r="F1" s="62" t="n"/>
     </row>
     <row r="2" ht="16.2" customHeight="1" thickBot="1">
-      <c r="A2" s="22" t="n"/>
-      <c r="B2" s="49" t="n"/>
-      <c r="C2" s="49" t="n"/>
-      <c r="D2" s="49" t="n"/>
-      <c r="E2" s="61" t="n"/>
-      <c r="F2" s="62" t="n"/>
+      <c r="A2" s="58" t="n"/>
+      <c r="B2" s="59" t="n"/>
+      <c r="C2" s="59" t="n"/>
+      <c r="D2" s="59" t="n"/>
+      <c r="E2" s="63" t="n"/>
+      <c r="F2" s="64" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="22" t="n"/>
-      <c r="B3" s="49" t="n"/>
-      <c r="C3" s="49" t="n"/>
-      <c r="D3" s="49" t="n"/>
-      <c r="E3" s="49" t="n"/>
+      <c r="A3" s="58" t="n"/>
+      <c r="B3" s="59" t="n"/>
+      <c r="C3" s="59" t="n"/>
+      <c r="D3" s="59" t="n"/>
+      <c r="E3" s="59" t="n"/>
       <c r="F3" s="29" t="inlineStr">
         <is>
-          <t>v1.0.1</t>
+          <t>v1.0.2</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="n"/>
-      <c r="B4" s="49" t="n"/>
-      <c r="C4" s="49" t="n"/>
-      <c r="D4" s="49" t="n"/>
-      <c r="E4" s="49" t="n"/>
-      <c r="F4" s="23" t="n"/>
+      <c r="A4" s="58" t="n"/>
+      <c r="B4" s="59" t="n"/>
+      <c r="C4" s="59" t="n"/>
+      <c r="D4" s="59" t="n"/>
+      <c r="E4" s="59" t="n"/>
+      <c r="F4" s="60" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="n"/>
+      <c r="A5" s="58" t="n"/>
       <c r="B5" s="48" t="inlineStr">
         <is>
           <t>Interlocking Program</t>
         </is>
       </c>
-      <c r="F5" s="23" t="n"/>
+      <c r="F5" s="60" t="n"/>
     </row>
     <row r="6" ht="14.4" customHeight="1">
       <c r="A6" s="24" t="n"/>
@@ -1240,94 +1250,92 @@
       <c r="F7" s="25" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="n"/>
-      <c r="B8" s="49" t="inlineStr">
-        <is>
-          <t>Cascais (CIS)</t>
-        </is>
-      </c>
-      <c r="F8" s="23" t="n"/>
+      <c r="A8" s="65" t="inlineStr">
+        <is>
+          <t>Cascais (NOT REAL DATA - FOR TESTING ONLY) (CIS)</t>
+        </is>
+      </c>
+      <c r="F8" s="66" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="n"/>
-      <c r="B9" s="49" t="inlineStr">
+      <c r="A9" s="65" t="inlineStr">
         <is>
           <t>Linha de Cascais</t>
         </is>
       </c>
-      <c r="F9" s="23" t="n"/>
+      <c r="F9" s="66" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="n"/>
-      <c r="B10" s="49" t="n"/>
-      <c r="C10" s="49" t="n"/>
-      <c r="D10" s="49" t="n"/>
-      <c r="E10" s="49" t="n"/>
-      <c r="F10" s="23" t="n"/>
+      <c r="A10" s="58" t="n"/>
+      <c r="B10" s="59" t="n"/>
+      <c r="C10" s="59" t="n"/>
+      <c r="D10" s="59" t="n"/>
+      <c r="E10" s="59" t="n"/>
+      <c r="F10" s="60" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="n"/>
-      <c r="B11" s="49" t="n"/>
-      <c r="C11" s="49" t="n"/>
-      <c r="D11" s="49" t="n"/>
-      <c r="E11" s="49" t="n"/>
-      <c r="F11" s="23" t="n"/>
+      <c r="A11" s="58" t="n"/>
+      <c r="B11" s="59" t="n"/>
+      <c r="C11" s="59" t="n"/>
+      <c r="D11" s="59" t="n"/>
+      <c r="E11" s="59" t="n"/>
+      <c r="F11" s="60" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="n"/>
-      <c r="B12" s="49" t="n"/>
-      <c r="C12" s="49" t="n"/>
-      <c r="D12" s="49" t="n"/>
-      <c r="E12" s="49" t="n"/>
-      <c r="F12" s="23" t="n"/>
+      <c r="A12" s="58" t="n"/>
+      <c r="B12" s="59" t="n"/>
+      <c r="C12" s="59" t="n"/>
+      <c r="D12" s="59" t="n"/>
+      <c r="E12" s="59" t="n"/>
+      <c r="F12" s="60" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="n"/>
-      <c r="B13" s="49" t="n"/>
-      <c r="C13" s="49" t="n"/>
-      <c r="D13" s="49" t="n"/>
-      <c r="E13" s="49" t="n"/>
-      <c r="F13" s="23" t="n"/>
+      <c r="A13" s="58" t="n"/>
+      <c r="B13" s="59" t="n"/>
+      <c r="C13" s="59" t="n"/>
+      <c r="D13" s="59" t="n"/>
+      <c r="E13" s="59" t="n"/>
+      <c r="F13" s="60" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="n"/>
-      <c r="B14" s="49" t="n"/>
-      <c r="C14" s="49" t="n"/>
-      <c r="D14" s="49" t="n"/>
-      <c r="E14" s="49" t="n"/>
-      <c r="F14" s="23" t="n"/>
+      <c r="A14" s="58" t="n"/>
+      <c r="B14" s="59" t="n"/>
+      <c r="C14" s="59" t="n"/>
+      <c r="D14" s="59" t="n"/>
+      <c r="E14" s="59" t="n"/>
+      <c r="F14" s="60" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="n"/>
-      <c r="B15" s="49" t="n"/>
-      <c r="C15" s="49" t="n"/>
-      <c r="D15" s="49" t="n"/>
-      <c r="E15" s="49" t="n"/>
-      <c r="F15" s="23" t="n"/>
+      <c r="A15" s="58" t="n"/>
+      <c r="B15" s="59" t="n"/>
+      <c r="C15" s="59" t="n"/>
+      <c r="D15" s="59" t="n"/>
+      <c r="E15" s="59" t="n"/>
+      <c r="F15" s="60" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="n"/>
-      <c r="B16" s="49" t="n"/>
-      <c r="C16" s="49" t="n"/>
-      <c r="D16" s="49" t="n"/>
-      <c r="E16" s="49" t="n"/>
-      <c r="F16" s="23" t="n"/>
+      <c r="A16" s="58" t="n"/>
+      <c r="B16" s="59" t="n"/>
+      <c r="C16" s="59" t="n"/>
+      <c r="D16" s="59" t="n"/>
+      <c r="E16" s="59" t="n"/>
+      <c r="F16" s="60" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="n"/>
-      <c r="B17" s="49" t="n"/>
-      <c r="C17" s="49" t="n"/>
-      <c r="D17" s="49" t="n"/>
-      <c r="E17" s="49" t="n"/>
-      <c r="F17" s="23" t="n"/>
+      <c r="A17" s="58" t="n"/>
+      <c r="B17" s="59" t="n"/>
+      <c r="C17" s="59" t="n"/>
+      <c r="D17" s="59" t="n"/>
+      <c r="E17" s="59" t="n"/>
+      <c r="F17" s="60" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="n"/>
-      <c r="B18" s="49" t="n"/>
-      <c r="C18" s="49" t="n"/>
-      <c r="D18" s="49" t="n"/>
-      <c r="E18" s="49" t="n"/>
-      <c r="F18" s="23" t="n"/>
+      <c r="A18" s="58" t="n"/>
+      <c r="B18" s="59" t="n"/>
+      <c r="C18" s="59" t="n"/>
+      <c r="D18" s="59" t="n"/>
+      <c r="E18" s="59" t="n"/>
+      <c r="F18" s="60" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
@@ -1335,11 +1343,11 @@
           <t>Diogo Luís</t>
         </is>
       </c>
-      <c r="B19" s="49" t="n"/>
-      <c r="C19" s="49" t="n"/>
-      <c r="D19" s="49" t="n"/>
-      <c r="E19" s="49" t="n"/>
-      <c r="F19" s="23" t="n"/>
+      <c r="B19" s="59" t="n"/>
+      <c r="C19" s="59" t="n"/>
+      <c r="D19" s="59" t="n"/>
+      <c r="E19" s="59" t="n"/>
+      <c r="F19" s="60" t="n"/>
     </row>
     <row r="20" ht="16.2" customHeight="1" thickBot="1">
       <c r="A20" s="31" t="inlineStr">
@@ -1355,9 +1363,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A8:F8"/>
     <mergeCell ref="B5:E6"/>
-    <mergeCell ref="B9:E9"/>
-    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="A9:F9"/>
     <mergeCell ref="E1:F2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1385,310 +1393,310 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B1" s="63" t="n"/>
-      <c r="C1" s="63" t="n"/>
-      <c r="D1" s="63" t="n"/>
-      <c r="E1" s="63" t="n"/>
-      <c r="F1" s="63" t="n"/>
-      <c r="G1" s="63" t="n"/>
-      <c r="H1" s="63" t="n"/>
-      <c r="I1" s="64" t="n"/>
-      <c r="J1" s="55" t="inlineStr">
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="67" t="n"/>
+      <c r="G1" s="67" t="n"/>
+      <c r="H1" s="67" t="n"/>
+      <c r="I1" s="68" t="n"/>
+      <c r="J1" s="54" t="inlineStr">
         <is>
           <t>Interlocking</t>
         </is>
       </c>
-      <c r="K1" s="65" t="n"/>
-      <c r="L1" s="65" t="n"/>
-      <c r="M1" s="65" t="n"/>
-      <c r="N1" s="65" t="n"/>
-      <c r="O1" s="65" t="n"/>
-      <c r="P1" s="65" t="n"/>
-      <c r="Q1" s="65" t="n"/>
-      <c r="R1" s="65" t="n"/>
-      <c r="S1" s="65" t="n"/>
-      <c r="T1" s="65" t="n"/>
-      <c r="U1" s="65" t="n"/>
-      <c r="V1" s="65" t="n"/>
-      <c r="W1" s="65" t="n"/>
-      <c r="X1" s="65" t="n"/>
-      <c r="Y1" s="65" t="n"/>
-      <c r="Z1" s="65" t="n"/>
-      <c r="AA1" s="66" t="n"/>
+      <c r="K1" s="69" t="n"/>
+      <c r="L1" s="69" t="n"/>
+      <c r="M1" s="69" t="n"/>
+      <c r="N1" s="69" t="n"/>
+      <c r="O1" s="69" t="n"/>
+      <c r="P1" s="69" t="n"/>
+      <c r="Q1" s="69" t="n"/>
+      <c r="R1" s="69" t="n"/>
+      <c r="S1" s="69" t="n"/>
+      <c r="T1" s="69" t="n"/>
+      <c r="U1" s="69" t="n"/>
+      <c r="V1" s="69" t="n"/>
+      <c r="W1" s="69" t="n"/>
+      <c r="X1" s="69" t="n"/>
+      <c r="Y1" s="69" t="n"/>
+      <c r="Z1" s="69" t="n"/>
+      <c r="AA1" s="70" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="67" t="n"/>
-      <c r="I2" s="68" t="n"/>
-      <c r="J2" s="50" t="inlineStr">
+      <c r="A2" s="71" t="n"/>
+      <c r="I2" s="72" t="n"/>
+      <c r="J2" s="49" t="inlineStr">
         <is>
           <t>Required Switches</t>
         </is>
       </c>
-      <c r="K2" s="69" t="n"/>
-      <c r="L2" s="69" t="n"/>
-      <c r="M2" s="69" t="n"/>
-      <c r="N2" s="69" t="n"/>
-      <c r="O2" s="69" t="n"/>
-      <c r="P2" s="69" t="n"/>
-      <c r="Q2" s="70" t="n"/>
-      <c r="R2" s="50" t="inlineStr">
+      <c r="K2" s="73" t="n"/>
+      <c r="L2" s="73" t="n"/>
+      <c r="M2" s="73" t="n"/>
+      <c r="N2" s="73" t="n"/>
+      <c r="O2" s="73" t="n"/>
+      <c r="P2" s="73" t="n"/>
+      <c r="Q2" s="74" t="n"/>
+      <c r="R2" s="49" t="inlineStr">
         <is>
           <t>Required Sections</t>
         </is>
       </c>
-      <c r="S2" s="69" t="n"/>
-      <c r="T2" s="69" t="n"/>
-      <c r="U2" s="69" t="n"/>
-      <c r="V2" s="69" t="n"/>
-      <c r="W2" s="69" t="n"/>
-      <c r="X2" s="69" t="n"/>
-      <c r="Y2" s="70" t="n"/>
-      <c r="Z2" s="50" t="inlineStr">
+      <c r="S2" s="73" t="n"/>
+      <c r="T2" s="73" t="n"/>
+      <c r="U2" s="73" t="n"/>
+      <c r="V2" s="73" t="n"/>
+      <c r="W2" s="73" t="n"/>
+      <c r="X2" s="73" t="n"/>
+      <c r="Y2" s="74" t="n"/>
+      <c r="Z2" s="49" t="inlineStr">
         <is>
           <t>Required Blocks</t>
         </is>
       </c>
-      <c r="AA2" s="71" t="n"/>
+      <c r="AA2" s="75" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="72" t="n"/>
-      <c r="B3" s="73" t="n"/>
-      <c r="C3" s="73" t="n"/>
-      <c r="D3" s="73" t="n"/>
-      <c r="E3" s="73" t="n"/>
-      <c r="F3" s="73" t="n"/>
-      <c r="G3" s="73" t="n"/>
-      <c r="H3" s="73" t="n"/>
-      <c r="I3" s="74" t="n"/>
-      <c r="J3" s="50" t="inlineStr">
+      <c r="A3" s="76" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="78" t="n"/>
+      <c r="J3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="K3" s="71" t="n"/>
-      <c r="L3" s="50" t="inlineStr">
+      <c r="K3" s="75" t="n"/>
+      <c r="L3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="M3" s="71" t="n"/>
-      <c r="N3" s="50" t="inlineStr">
+      <c r="M3" s="75" t="n"/>
+      <c r="N3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="O3" s="69" t="n"/>
-      <c r="P3" s="69" t="n"/>
-      <c r="Q3" s="70" t="n"/>
-      <c r="R3" s="50" t="inlineStr">
+      <c r="O3" s="73" t="n"/>
+      <c r="P3" s="73" t="n"/>
+      <c r="Q3" s="74" t="n"/>
+      <c r="R3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="S3" s="50" t="inlineStr">
+      <c r="S3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="T3" s="50" t="inlineStr">
+      <c r="T3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="U3" s="69" t="n"/>
-      <c r="V3" s="69" t="n"/>
-      <c r="W3" s="69" t="n"/>
-      <c r="X3" s="69" t="n"/>
-      <c r="Y3" s="70" t="n"/>
-      <c r="Z3" s="75" t="n"/>
-      <c r="AA3" s="68" t="n"/>
+      <c r="U3" s="73" t="n"/>
+      <c r="V3" s="73" t="n"/>
+      <c r="W3" s="73" t="n"/>
+      <c r="X3" s="73" t="n"/>
+      <c r="Y3" s="74" t="n"/>
+      <c r="Z3" s="79" t="n"/>
+      <c r="AA3" s="72" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="51" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="C4" s="70" t="n"/>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="C4" s="74" t="n"/>
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="E4" s="70" t="n"/>
-      <c r="F4" s="52" t="inlineStr">
+      <c r="E4" s="74" t="n"/>
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="G4" s="52" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="H4" s="70" t="n"/>
-      <c r="I4" s="52" t="inlineStr">
+      <c r="H4" s="74" t="n"/>
+      <c r="I4" s="51" t="inlineStr">
         <is>
           <t>Obs.</t>
         </is>
       </c>
-      <c r="J4" s="76" t="n"/>
-      <c r="K4" s="74" t="n"/>
-      <c r="L4" s="76" t="n"/>
-      <c r="M4" s="74" t="n"/>
-      <c r="N4" s="50" t="inlineStr">
+      <c r="J4" s="80" t="n"/>
+      <c r="K4" s="78" t="n"/>
+      <c r="L4" s="80" t="n"/>
+      <c r="M4" s="78" t="n"/>
+      <c r="N4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="O4" s="70" t="n"/>
-      <c r="P4" s="50" t="inlineStr">
+      <c r="O4" s="74" t="n"/>
+      <c r="P4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="Q4" s="70" t="n"/>
-      <c r="R4" s="77" t="n"/>
-      <c r="S4" s="77" t="n"/>
-      <c r="T4" s="50" t="inlineStr">
+      <c r="Q4" s="74" t="n"/>
+      <c r="R4" s="81" t="n"/>
+      <c r="S4" s="81" t="n"/>
+      <c r="T4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="U4" s="69" t="n"/>
-      <c r="V4" s="70" t="n"/>
-      <c r="W4" s="50" t="inlineStr">
+      <c r="U4" s="73" t="n"/>
+      <c r="V4" s="74" t="n"/>
+      <c r="W4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="X4" s="69" t="n"/>
-      <c r="Y4" s="70" t="n"/>
-      <c r="Z4" s="76" t="n"/>
-      <c r="AA4" s="74" t="n"/>
+      <c r="X4" s="73" t="n"/>
+      <c r="Y4" s="74" t="n"/>
+      <c r="Z4" s="80" t="n"/>
+      <c r="AA4" s="78" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="78" t="n"/>
-      <c r="B5" s="52" t="inlineStr">
+      <c r="A5" s="82" t="n"/>
+      <c r="B5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="C5" s="52" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D5" s="52" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="E5" s="52" t="inlineStr">
+      <c r="E5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F5" s="79" t="n"/>
-      <c r="G5" s="52" t="inlineStr">
+      <c r="F5" s="83" t="n"/>
+      <c r="G5" s="51" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="H5" s="52" t="inlineStr">
+      <c r="H5" s="51" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="I5" s="79" t="n"/>
-      <c r="J5" s="50" t="inlineStr">
+      <c r="I5" s="83" t="n"/>
+      <c r="J5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="K5" s="50" t="inlineStr">
+      <c r="K5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="L5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="M5" s="50" t="inlineStr">
+      <c r="M5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="N5" s="50" t="inlineStr">
+      <c r="N5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="O5" s="50" t="inlineStr">
+      <c r="O5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="P5" s="50" t="inlineStr">
+      <c r="P5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q5" s="50" t="inlineStr">
+      <c r="Q5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="R5" s="79" t="n"/>
-      <c r="S5" s="79" t="n"/>
-      <c r="T5" s="50" t="inlineStr">
+      <c r="R5" s="83" t="n"/>
+      <c r="S5" s="83" t="n"/>
+      <c r="T5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="U5" s="50" t="inlineStr">
+      <c r="U5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="V5" s="50" t="inlineStr">
+      <c r="V5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="W5" s="50" t="inlineStr">
+      <c r="W5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="X5" s="50" t="inlineStr">
+      <c r="X5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="Y5" s="50" t="inlineStr">
+      <c r="Y5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="Z5" s="50" t="inlineStr">
+      <c r="Z5" s="49" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="AA5" s="57" t="inlineStr">
+      <c r="AA5" s="56" t="inlineStr">
         <is>
           <t>Down</t>
         </is>
@@ -1745,7 +1753,7 @@
       </c>
       <c r="O6" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P6" s="11" t="inlineStr"/>
@@ -1816,7 +1824,7 @@
       </c>
       <c r="O7" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P7" s="11" t="inlineStr"/>
@@ -1866,7 +1874,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>1II, 3I, 7, 13</t>
+          <t>1II, 3I, 7, 15</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
@@ -1890,7 +1898,7 @@
       <c r="Q8" s="12" t="inlineStr"/>
       <c r="R8" s="11" t="inlineStr">
         <is>
-          <t>1II, A1, 3I, 7, 11/13</t>
+          <t>1II, A1, 3I, 7, 11/15</t>
         </is>
       </c>
       <c r="S8" s="12" t="inlineStr"/>
@@ -1937,7 +1945,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>1II, 3I, 7, 13</t>
+          <t>1II, 3I, 7, 15</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -2004,7 +2012,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>1II, 3I, 7, 11, 13</t>
+          <t>1II, 3I, 7, 11, 15</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr"/>
@@ -2024,7 +2032,7 @@
       <c r="Q10" s="12" t="inlineStr"/>
       <c r="R10" s="11" t="inlineStr">
         <is>
-          <t>1II, A1, 3I, 7, 11/13</t>
+          <t>1II, A1, 3I, 7, 11/15</t>
         </is>
       </c>
       <c r="S10" s="12" t="inlineStr"/>
@@ -2071,7 +2079,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>1II, 3I, 7, 11, 13</t>
+          <t>1II, 3I, 7, 11, 15</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr"/>
@@ -2151,7 +2159,7 @@
       </c>
       <c r="O12" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P12" s="11" t="inlineStr"/>
@@ -2164,7 +2172,7 @@
       <c r="S12" s="12" t="inlineStr"/>
       <c r="T12" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U12" s="12" t="inlineStr"/>
@@ -2226,7 +2234,7 @@
       </c>
       <c r="O13" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P13" s="11" t="inlineStr"/>
@@ -2235,7 +2243,7 @@
       <c r="S13" s="12" t="inlineStr"/>
       <c r="T13" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U13" s="12" t="inlineStr"/>
@@ -2297,7 +2305,7 @@
       </c>
       <c r="O14" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P14" s="11" t="inlineStr"/>
@@ -2310,7 +2318,7 @@
       <c r="S14" s="12" t="inlineStr"/>
       <c r="T14" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U14" s="12" t="inlineStr"/>
@@ -2372,7 +2380,7 @@
       </c>
       <c r="O15" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P15" s="11" t="inlineStr"/>
@@ -2381,7 +2389,7 @@
       <c r="S15" s="12" t="inlineStr"/>
       <c r="T15" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U15" s="12" t="inlineStr"/>
@@ -5051,310 +5059,310 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B1" s="63" t="n"/>
-      <c r="C1" s="63" t="n"/>
-      <c r="D1" s="63" t="n"/>
-      <c r="E1" s="63" t="n"/>
-      <c r="F1" s="63" t="n"/>
-      <c r="G1" s="63" t="n"/>
-      <c r="H1" s="63" t="n"/>
-      <c r="I1" s="64" t="n"/>
-      <c r="J1" s="55" t="inlineStr">
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="67" t="n"/>
+      <c r="G1" s="67" t="n"/>
+      <c r="H1" s="67" t="n"/>
+      <c r="I1" s="68" t="n"/>
+      <c r="J1" s="54" t="inlineStr">
         <is>
           <t>Interlocking</t>
         </is>
       </c>
-      <c r="K1" s="65" t="n"/>
-      <c r="L1" s="65" t="n"/>
-      <c r="M1" s="65" t="n"/>
-      <c r="N1" s="65" t="n"/>
-      <c r="O1" s="65" t="n"/>
-      <c r="P1" s="65" t="n"/>
-      <c r="Q1" s="65" t="n"/>
-      <c r="R1" s="65" t="n"/>
-      <c r="S1" s="65" t="n"/>
-      <c r="T1" s="65" t="n"/>
-      <c r="U1" s="65" t="n"/>
-      <c r="V1" s="65" t="n"/>
-      <c r="W1" s="65" t="n"/>
-      <c r="X1" s="65" t="n"/>
-      <c r="Y1" s="65" t="n"/>
-      <c r="Z1" s="65" t="n"/>
-      <c r="AA1" s="66" t="n"/>
+      <c r="K1" s="69" t="n"/>
+      <c r="L1" s="69" t="n"/>
+      <c r="M1" s="69" t="n"/>
+      <c r="N1" s="69" t="n"/>
+      <c r="O1" s="69" t="n"/>
+      <c r="P1" s="69" t="n"/>
+      <c r="Q1" s="69" t="n"/>
+      <c r="R1" s="69" t="n"/>
+      <c r="S1" s="69" t="n"/>
+      <c r="T1" s="69" t="n"/>
+      <c r="U1" s="69" t="n"/>
+      <c r="V1" s="69" t="n"/>
+      <c r="W1" s="69" t="n"/>
+      <c r="X1" s="69" t="n"/>
+      <c r="Y1" s="69" t="n"/>
+      <c r="Z1" s="69" t="n"/>
+      <c r="AA1" s="70" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="67" t="n"/>
-      <c r="I2" s="68" t="n"/>
-      <c r="J2" s="50" t="inlineStr">
+      <c r="A2" s="71" t="n"/>
+      <c r="I2" s="72" t="n"/>
+      <c r="J2" s="49" t="inlineStr">
         <is>
           <t>Required Switches</t>
         </is>
       </c>
-      <c r="K2" s="69" t="n"/>
-      <c r="L2" s="69" t="n"/>
-      <c r="M2" s="69" t="n"/>
-      <c r="N2" s="69" t="n"/>
-      <c r="O2" s="69" t="n"/>
-      <c r="P2" s="69" t="n"/>
-      <c r="Q2" s="70" t="n"/>
-      <c r="R2" s="50" t="inlineStr">
+      <c r="K2" s="73" t="n"/>
+      <c r="L2" s="73" t="n"/>
+      <c r="M2" s="73" t="n"/>
+      <c r="N2" s="73" t="n"/>
+      <c r="O2" s="73" t="n"/>
+      <c r="P2" s="73" t="n"/>
+      <c r="Q2" s="74" t="n"/>
+      <c r="R2" s="49" t="inlineStr">
         <is>
           <t>Required Sections</t>
         </is>
       </c>
-      <c r="S2" s="69" t="n"/>
-      <c r="T2" s="69" t="n"/>
-      <c r="U2" s="69" t="n"/>
-      <c r="V2" s="69" t="n"/>
-      <c r="W2" s="69" t="n"/>
-      <c r="X2" s="69" t="n"/>
-      <c r="Y2" s="70" t="n"/>
-      <c r="Z2" s="50" t="inlineStr">
+      <c r="S2" s="73" t="n"/>
+      <c r="T2" s="73" t="n"/>
+      <c r="U2" s="73" t="n"/>
+      <c r="V2" s="73" t="n"/>
+      <c r="W2" s="73" t="n"/>
+      <c r="X2" s="73" t="n"/>
+      <c r="Y2" s="74" t="n"/>
+      <c r="Z2" s="49" t="inlineStr">
         <is>
           <t>Required Blocks</t>
         </is>
       </c>
-      <c r="AA2" s="71" t="n"/>
+      <c r="AA2" s="75" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="72" t="n"/>
-      <c r="B3" s="73" t="n"/>
-      <c r="C3" s="73" t="n"/>
-      <c r="D3" s="73" t="n"/>
-      <c r="E3" s="73" t="n"/>
-      <c r="F3" s="73" t="n"/>
-      <c r="G3" s="73" t="n"/>
-      <c r="H3" s="73" t="n"/>
-      <c r="I3" s="74" t="n"/>
-      <c r="J3" s="50" t="inlineStr">
+      <c r="A3" s="76" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="78" t="n"/>
+      <c r="J3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="K3" s="71" t="n"/>
-      <c r="L3" s="50" t="inlineStr">
+      <c r="K3" s="75" t="n"/>
+      <c r="L3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="M3" s="71" t="n"/>
-      <c r="N3" s="50" t="inlineStr">
+      <c r="M3" s="75" t="n"/>
+      <c r="N3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="O3" s="69" t="n"/>
-      <c r="P3" s="69" t="n"/>
-      <c r="Q3" s="70" t="n"/>
-      <c r="R3" s="50" t="inlineStr">
+      <c r="O3" s="73" t="n"/>
+      <c r="P3" s="73" t="n"/>
+      <c r="Q3" s="74" t="n"/>
+      <c r="R3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="S3" s="50" t="inlineStr">
+      <c r="S3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="T3" s="50" t="inlineStr">
+      <c r="T3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="U3" s="69" t="n"/>
-      <c r="V3" s="69" t="n"/>
-      <c r="W3" s="69" t="n"/>
-      <c r="X3" s="69" t="n"/>
-      <c r="Y3" s="70" t="n"/>
-      <c r="Z3" s="75" t="n"/>
-      <c r="AA3" s="68" t="n"/>
+      <c r="U3" s="73" t="n"/>
+      <c r="V3" s="73" t="n"/>
+      <c r="W3" s="73" t="n"/>
+      <c r="X3" s="73" t="n"/>
+      <c r="Y3" s="74" t="n"/>
+      <c r="Z3" s="79" t="n"/>
+      <c r="AA3" s="72" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="51" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="C4" s="70" t="n"/>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="C4" s="74" t="n"/>
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="E4" s="70" t="n"/>
-      <c r="F4" s="52" t="inlineStr">
+      <c r="E4" s="74" t="n"/>
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="G4" s="52" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="H4" s="70" t="n"/>
-      <c r="I4" s="52" t="inlineStr">
+      <c r="H4" s="74" t="n"/>
+      <c r="I4" s="51" t="inlineStr">
         <is>
           <t>Obs.</t>
         </is>
       </c>
-      <c r="J4" s="76" t="n"/>
-      <c r="K4" s="74" t="n"/>
-      <c r="L4" s="76" t="n"/>
-      <c r="M4" s="74" t="n"/>
-      <c r="N4" s="50" t="inlineStr">
+      <c r="J4" s="80" t="n"/>
+      <c r="K4" s="78" t="n"/>
+      <c r="L4" s="80" t="n"/>
+      <c r="M4" s="78" t="n"/>
+      <c r="N4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="O4" s="70" t="n"/>
-      <c r="P4" s="50" t="inlineStr">
+      <c r="O4" s="74" t="n"/>
+      <c r="P4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="Q4" s="70" t="n"/>
-      <c r="R4" s="77" t="n"/>
-      <c r="S4" s="77" t="n"/>
-      <c r="T4" s="50" t="inlineStr">
+      <c r="Q4" s="74" t="n"/>
+      <c r="R4" s="81" t="n"/>
+      <c r="S4" s="81" t="n"/>
+      <c r="T4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="U4" s="69" t="n"/>
-      <c r="V4" s="70" t="n"/>
-      <c r="W4" s="50" t="inlineStr">
+      <c r="U4" s="73" t="n"/>
+      <c r="V4" s="74" t="n"/>
+      <c r="W4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="X4" s="69" t="n"/>
-      <c r="Y4" s="70" t="n"/>
-      <c r="Z4" s="76" t="n"/>
-      <c r="AA4" s="74" t="n"/>
+      <c r="X4" s="73" t="n"/>
+      <c r="Y4" s="74" t="n"/>
+      <c r="Z4" s="80" t="n"/>
+      <c r="AA4" s="78" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="78" t="n"/>
-      <c r="B5" s="52" t="inlineStr">
+      <c r="A5" s="82" t="n"/>
+      <c r="B5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="C5" s="52" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D5" s="52" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="E5" s="52" t="inlineStr">
+      <c r="E5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F5" s="79" t="n"/>
-      <c r="G5" s="52" t="inlineStr">
+      <c r="F5" s="83" t="n"/>
+      <c r="G5" s="51" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="H5" s="52" t="inlineStr">
+      <c r="H5" s="51" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="I5" s="79" t="n"/>
-      <c r="J5" s="50" t="inlineStr">
+      <c r="I5" s="83" t="n"/>
+      <c r="J5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="K5" s="50" t="inlineStr">
+      <c r="K5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="L5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="M5" s="50" t="inlineStr">
+      <c r="M5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="N5" s="50" t="inlineStr">
+      <c r="N5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="O5" s="50" t="inlineStr">
+      <c r="O5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="P5" s="50" t="inlineStr">
+      <c r="P5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q5" s="50" t="inlineStr">
+      <c r="Q5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="R5" s="79" t="n"/>
-      <c r="S5" s="79" t="n"/>
-      <c r="T5" s="50" t="inlineStr">
+      <c r="R5" s="83" t="n"/>
+      <c r="S5" s="83" t="n"/>
+      <c r="T5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="U5" s="50" t="inlineStr">
+      <c r="U5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="V5" s="50" t="inlineStr">
+      <c r="V5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="W5" s="50" t="inlineStr">
+      <c r="W5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="X5" s="50" t="inlineStr">
+      <c r="X5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="Y5" s="50" t="inlineStr">
+      <c r="Y5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="Z5" s="50" t="inlineStr">
+      <c r="Z5" s="49" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="AA5" s="57" t="inlineStr">
+      <c r="AA5" s="56" t="inlineStr">
         <is>
           <t>Down</t>
         </is>
@@ -5366,7 +5374,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -5392,13 +5400,13 @@
       <c r="G6" s="10" t="inlineStr"/>
       <c r="H6" s="9" t="inlineStr">
         <is>
-          <t>13+</t>
+          <t>15+</t>
         </is>
       </c>
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>13, 7, 3I</t>
+          <t>15, 7, 3I</t>
         </is>
       </c>
       <c r="K6" s="12" t="inlineStr">
@@ -5418,7 +5426,7 @@
       <c r="Q6" s="12" t="inlineStr"/>
       <c r="R6" s="11" t="inlineStr">
         <is>
-          <t>11/13, 7, 3I, A1, 1II, 1I, D1</t>
+          <t>11/15, 7, 3I, A1, 1II, 1I, B1</t>
         </is>
       </c>
       <c r="S6" s="12" t="inlineStr"/>
@@ -5449,7 +5457,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -5475,7 +5483,7 @@
       <c r="G7" s="10" t="inlineStr"/>
       <c r="H7" s="9" t="inlineStr">
         <is>
-          <t>13-</t>
+          <t>15-</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr"/>
@@ -5486,7 +5494,7 @@
       </c>
       <c r="K7" s="12" t="inlineStr">
         <is>
-          <t>11, 13</t>
+          <t>11, 15</t>
         </is>
       </c>
       <c r="L7" s="11" t="inlineStr"/>
@@ -5505,7 +5513,7 @@
       <c r="Q7" s="12" t="inlineStr"/>
       <c r="R7" s="11" t="inlineStr">
         <is>
-          <t>11/13, 3II/5, 1I, D1</t>
+          <t>11/15, 3II/5, 1I, B1</t>
         </is>
       </c>
       <c r="S7" s="12" t="inlineStr"/>
@@ -5532,7 +5540,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -5558,13 +5566,13 @@
       <c r="G8" s="10" t="inlineStr"/>
       <c r="H8" s="9" t="inlineStr">
         <is>
-          <t>13+</t>
+          <t>15+</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>13, 7, 3I</t>
+          <t>15, 7, 3I</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
@@ -5611,7 +5619,7 @@
       </c>
       <c r="B9" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C9" s="10" t="inlineStr">
@@ -5637,7 +5645,7 @@
       <c r="G9" s="10" t="inlineStr"/>
       <c r="H9" s="9" t="inlineStr">
         <is>
-          <t>13-</t>
+          <t>15-</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr"/>
@@ -5648,7 +5656,7 @@
       </c>
       <c r="K9" s="12" t="inlineStr">
         <is>
-          <t>11, 13</t>
+          <t>11, 15</t>
         </is>
       </c>
       <c r="L9" s="11" t="inlineStr"/>
@@ -5716,13 +5724,13 @@
       <c r="G10" s="10" t="inlineStr"/>
       <c r="H10" s="9" t="inlineStr">
         <is>
-          <t>13+</t>
+          <t>15+</t>
         </is>
       </c>
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>11, 13, 7, 3I</t>
+          <t>11, 15, 7, 3I</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
@@ -5742,7 +5750,7 @@
       <c r="Q10" s="12" t="inlineStr"/>
       <c r="R10" s="11" t="inlineStr">
         <is>
-          <t>11/13, 7, 3I, A1, 1II, 1I, D1</t>
+          <t>11/15, 7, 3I, A1, 1II, 1I, B1</t>
         </is>
       </c>
       <c r="S10" s="12" t="inlineStr"/>
@@ -5799,7 +5807,7 @@
       <c r="G11" s="10" t="inlineStr"/>
       <c r="H11" s="9" t="inlineStr">
         <is>
-          <t>13-</t>
+          <t>15-</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr"/>
@@ -5810,7 +5818,7 @@
       </c>
       <c r="K11" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="L11" s="11" t="inlineStr"/>
@@ -5829,7 +5837,7 @@
       <c r="Q11" s="12" t="inlineStr"/>
       <c r="R11" s="11" t="inlineStr">
         <is>
-          <t>11/13, 3II/5, 1I, D1</t>
+          <t>11/15, 3II/5, 1I, B1</t>
         </is>
       </c>
       <c r="S11" s="12" t="inlineStr"/>
@@ -5882,13 +5890,13 @@
       <c r="G12" s="10" t="inlineStr"/>
       <c r="H12" s="9" t="inlineStr">
         <is>
-          <t>13+</t>
+          <t>15+</t>
         </is>
       </c>
       <c r="I12" s="10" t="inlineStr"/>
       <c r="J12" s="11" t="inlineStr">
         <is>
-          <t>11, 13, 7, 3I</t>
+          <t>11, 15, 7, 3I</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
@@ -5961,7 +5969,7 @@
       <c r="G13" s="10" t="inlineStr"/>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>13-</t>
+          <t>15-</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr"/>
@@ -5972,7 +5980,7 @@
       </c>
       <c r="K13" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="L13" s="11" t="inlineStr"/>
@@ -6058,7 +6066,7 @@
       <c r="M14" s="12" t="inlineStr"/>
       <c r="N14" s="11" t="inlineStr">
         <is>
-          <t>13, 3I, 1II</t>
+          <t>15, 3I, 1II</t>
         </is>
       </c>
       <c r="O14" s="12" t="inlineStr"/>
@@ -6066,7 +6074,7 @@
       <c r="Q14" s="12" t="inlineStr"/>
       <c r="R14" s="11" t="inlineStr">
         <is>
-          <t>9, 3II/5, 1I, D1</t>
+          <t>9, 3II/5, 1I, B1</t>
         </is>
       </c>
       <c r="S14" s="12" t="inlineStr"/>
@@ -6133,7 +6141,7 @@
       <c r="M15" s="12" t="inlineStr"/>
       <c r="N15" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O15" s="12" t="inlineStr">
@@ -6145,7 +6153,7 @@
       <c r="Q15" s="12" t="inlineStr"/>
       <c r="R15" s="11" t="inlineStr">
         <is>
-          <t>9, 3II/5, 3I, A1, 1II, 1I, D1</t>
+          <t>9, 3II/5, 3I, A1, 1II, 1I, B1</t>
         </is>
       </c>
       <c r="S15" s="12" t="inlineStr"/>
@@ -6156,7 +6164,7 @@
       </c>
       <c r="U15" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V15" s="11" t="inlineStr"/>
@@ -6220,7 +6228,7 @@
       <c r="M16" s="12" t="inlineStr"/>
       <c r="N16" s="11" t="inlineStr">
         <is>
-          <t>13, 3I, 1II</t>
+          <t>15, 3I, 1II</t>
         </is>
       </c>
       <c r="O16" s="12" t="inlineStr"/>
@@ -6291,7 +6299,7 @@
       <c r="M17" s="12" t="inlineStr"/>
       <c r="N17" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O17" s="12" t="inlineStr">
@@ -6310,7 +6318,7 @@
       </c>
       <c r="U17" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V17" s="11" t="inlineStr"/>
@@ -6374,7 +6382,7 @@
       <c r="M18" s="12" t="inlineStr"/>
       <c r="N18" s="11" t="inlineStr">
         <is>
-          <t>13, 3I, 1II</t>
+          <t>15, 3I, 1II</t>
         </is>
       </c>
       <c r="O18" s="12" t="inlineStr"/>
@@ -6382,7 +6390,7 @@
       <c r="Q18" s="12" t="inlineStr"/>
       <c r="R18" s="11" t="inlineStr">
         <is>
-          <t>9, 3II/5, 1I, D1</t>
+          <t>9, 3II/5, 1I, B1</t>
         </is>
       </c>
       <c r="S18" s="12" t="inlineStr"/>
@@ -6445,7 +6453,7 @@
       <c r="M19" s="12" t="inlineStr"/>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O19" s="12" t="inlineStr">
@@ -6457,7 +6465,7 @@
       <c r="Q19" s="12" t="inlineStr"/>
       <c r="R19" s="11" t="inlineStr">
         <is>
-          <t>9, 3II/5, 3I, A1, 1II, 1I, D1</t>
+          <t>9, 3II/5, 3I, A1, 1II, 1I, B1</t>
         </is>
       </c>
       <c r="S19" s="12" t="inlineStr"/>
@@ -6468,7 +6476,7 @@
       </c>
       <c r="U19" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V19" s="11" t="inlineStr"/>
@@ -6532,7 +6540,7 @@
       <c r="M20" s="12" t="inlineStr"/>
       <c r="N20" s="11" t="inlineStr">
         <is>
-          <t>13, 3I, 1II</t>
+          <t>15, 3I, 1II</t>
         </is>
       </c>
       <c r="O20" s="12" t="inlineStr"/>
@@ -6599,7 +6607,7 @@
       <c r="M21" s="12" t="inlineStr"/>
       <c r="N21" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O21" s="12" t="inlineStr">
@@ -6618,7 +6626,7 @@
       </c>
       <c r="U21" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V21" s="11" t="inlineStr"/>
@@ -9117,310 +9125,310 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B1" s="63" t="n"/>
-      <c r="C1" s="63" t="n"/>
-      <c r="D1" s="63" t="n"/>
-      <c r="E1" s="63" t="n"/>
-      <c r="F1" s="63" t="n"/>
-      <c r="G1" s="63" t="n"/>
-      <c r="H1" s="63" t="n"/>
-      <c r="I1" s="64" t="n"/>
-      <c r="J1" s="55" t="inlineStr">
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="67" t="n"/>
+      <c r="G1" s="67" t="n"/>
+      <c r="H1" s="67" t="n"/>
+      <c r="I1" s="68" t="n"/>
+      <c r="J1" s="54" t="inlineStr">
         <is>
           <t>Interlocking</t>
         </is>
       </c>
-      <c r="K1" s="65" t="n"/>
-      <c r="L1" s="65" t="n"/>
-      <c r="M1" s="65" t="n"/>
-      <c r="N1" s="65" t="n"/>
-      <c r="O1" s="65" t="n"/>
-      <c r="P1" s="65" t="n"/>
-      <c r="Q1" s="65" t="n"/>
-      <c r="R1" s="65" t="n"/>
-      <c r="S1" s="65" t="n"/>
-      <c r="T1" s="65" t="n"/>
-      <c r="U1" s="65" t="n"/>
-      <c r="V1" s="65" t="n"/>
-      <c r="W1" s="65" t="n"/>
-      <c r="X1" s="65" t="n"/>
-      <c r="Y1" s="65" t="n"/>
-      <c r="Z1" s="65" t="n"/>
-      <c r="AA1" s="66" t="n"/>
+      <c r="K1" s="69" t="n"/>
+      <c r="L1" s="69" t="n"/>
+      <c r="M1" s="69" t="n"/>
+      <c r="N1" s="69" t="n"/>
+      <c r="O1" s="69" t="n"/>
+      <c r="P1" s="69" t="n"/>
+      <c r="Q1" s="69" t="n"/>
+      <c r="R1" s="69" t="n"/>
+      <c r="S1" s="69" t="n"/>
+      <c r="T1" s="69" t="n"/>
+      <c r="U1" s="69" t="n"/>
+      <c r="V1" s="69" t="n"/>
+      <c r="W1" s="69" t="n"/>
+      <c r="X1" s="69" t="n"/>
+      <c r="Y1" s="69" t="n"/>
+      <c r="Z1" s="69" t="n"/>
+      <c r="AA1" s="70" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="67" t="n"/>
-      <c r="I2" s="68" t="n"/>
-      <c r="J2" s="50" t="inlineStr">
+      <c r="A2" s="71" t="n"/>
+      <c r="I2" s="72" t="n"/>
+      <c r="J2" s="49" t="inlineStr">
         <is>
           <t>Required Switches</t>
         </is>
       </c>
-      <c r="K2" s="69" t="n"/>
-      <c r="L2" s="69" t="n"/>
-      <c r="M2" s="69" t="n"/>
-      <c r="N2" s="69" t="n"/>
-      <c r="O2" s="69" t="n"/>
-      <c r="P2" s="69" t="n"/>
-      <c r="Q2" s="70" t="n"/>
-      <c r="R2" s="50" t="inlineStr">
+      <c r="K2" s="73" t="n"/>
+      <c r="L2" s="73" t="n"/>
+      <c r="M2" s="73" t="n"/>
+      <c r="N2" s="73" t="n"/>
+      <c r="O2" s="73" t="n"/>
+      <c r="P2" s="73" t="n"/>
+      <c r="Q2" s="74" t="n"/>
+      <c r="R2" s="49" t="inlineStr">
         <is>
           <t>Required Sections</t>
         </is>
       </c>
-      <c r="S2" s="69" t="n"/>
-      <c r="T2" s="69" t="n"/>
-      <c r="U2" s="69" t="n"/>
-      <c r="V2" s="69" t="n"/>
-      <c r="W2" s="69" t="n"/>
-      <c r="X2" s="69" t="n"/>
-      <c r="Y2" s="70" t="n"/>
-      <c r="Z2" s="50" t="inlineStr">
+      <c r="S2" s="73" t="n"/>
+      <c r="T2" s="73" t="n"/>
+      <c r="U2" s="73" t="n"/>
+      <c r="V2" s="73" t="n"/>
+      <c r="W2" s="73" t="n"/>
+      <c r="X2" s="73" t="n"/>
+      <c r="Y2" s="74" t="n"/>
+      <c r="Z2" s="49" t="inlineStr">
         <is>
           <t>Required Blocks</t>
         </is>
       </c>
-      <c r="AA2" s="71" t="n"/>
+      <c r="AA2" s="75" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="72" t="n"/>
-      <c r="B3" s="73" t="n"/>
-      <c r="C3" s="73" t="n"/>
-      <c r="D3" s="73" t="n"/>
-      <c r="E3" s="73" t="n"/>
-      <c r="F3" s="73" t="n"/>
-      <c r="G3" s="73" t="n"/>
-      <c r="H3" s="73" t="n"/>
-      <c r="I3" s="74" t="n"/>
-      <c r="J3" s="50" t="inlineStr">
+      <c r="A3" s="76" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="78" t="n"/>
+      <c r="J3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="K3" s="71" t="n"/>
-      <c r="L3" s="50" t="inlineStr">
+      <c r="K3" s="75" t="n"/>
+      <c r="L3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="M3" s="71" t="n"/>
-      <c r="N3" s="50" t="inlineStr">
+      <c r="M3" s="75" t="n"/>
+      <c r="N3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="O3" s="69" t="n"/>
-      <c r="P3" s="69" t="n"/>
-      <c r="Q3" s="70" t="n"/>
-      <c r="R3" s="50" t="inlineStr">
+      <c r="O3" s="73" t="n"/>
+      <c r="P3" s="73" t="n"/>
+      <c r="Q3" s="74" t="n"/>
+      <c r="R3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="S3" s="50" t="inlineStr">
+      <c r="S3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="T3" s="50" t="inlineStr">
+      <c r="T3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="U3" s="69" t="n"/>
-      <c r="V3" s="69" t="n"/>
-      <c r="W3" s="69" t="n"/>
-      <c r="X3" s="69" t="n"/>
-      <c r="Y3" s="70" t="n"/>
-      <c r="Z3" s="75" t="n"/>
-      <c r="AA3" s="68" t="n"/>
+      <c r="U3" s="73" t="n"/>
+      <c r="V3" s="73" t="n"/>
+      <c r="W3" s="73" t="n"/>
+      <c r="X3" s="73" t="n"/>
+      <c r="Y3" s="74" t="n"/>
+      <c r="Z3" s="79" t="n"/>
+      <c r="AA3" s="72" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="51" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="C4" s="70" t="n"/>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="C4" s="74" t="n"/>
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="E4" s="70" t="n"/>
-      <c r="F4" s="52" t="inlineStr">
+      <c r="E4" s="74" t="n"/>
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="G4" s="52" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="H4" s="70" t="n"/>
-      <c r="I4" s="52" t="inlineStr">
+      <c r="H4" s="74" t="n"/>
+      <c r="I4" s="51" t="inlineStr">
         <is>
           <t>Obs.</t>
         </is>
       </c>
-      <c r="J4" s="76" t="n"/>
-      <c r="K4" s="74" t="n"/>
-      <c r="L4" s="76" t="n"/>
-      <c r="M4" s="74" t="n"/>
-      <c r="N4" s="50" t="inlineStr">
+      <c r="J4" s="80" t="n"/>
+      <c r="K4" s="78" t="n"/>
+      <c r="L4" s="80" t="n"/>
+      <c r="M4" s="78" t="n"/>
+      <c r="N4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="O4" s="70" t="n"/>
-      <c r="P4" s="50" t="inlineStr">
+      <c r="O4" s="74" t="n"/>
+      <c r="P4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="Q4" s="70" t="n"/>
-      <c r="R4" s="77" t="n"/>
-      <c r="S4" s="77" t="n"/>
-      <c r="T4" s="50" t="inlineStr">
+      <c r="Q4" s="74" t="n"/>
+      <c r="R4" s="81" t="n"/>
+      <c r="S4" s="81" t="n"/>
+      <c r="T4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="U4" s="69" t="n"/>
-      <c r="V4" s="70" t="n"/>
-      <c r="W4" s="50" t="inlineStr">
+      <c r="U4" s="73" t="n"/>
+      <c r="V4" s="74" t="n"/>
+      <c r="W4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="X4" s="69" t="n"/>
-      <c r="Y4" s="70" t="n"/>
-      <c r="Z4" s="76" t="n"/>
-      <c r="AA4" s="74" t="n"/>
+      <c r="X4" s="73" t="n"/>
+      <c r="Y4" s="74" t="n"/>
+      <c r="Z4" s="80" t="n"/>
+      <c r="AA4" s="78" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="78" t="n"/>
-      <c r="B5" s="52" t="inlineStr">
+      <c r="A5" s="82" t="n"/>
+      <c r="B5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="C5" s="52" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D5" s="52" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="E5" s="52" t="inlineStr">
+      <c r="E5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F5" s="79" t="n"/>
-      <c r="G5" s="52" t="inlineStr">
+      <c r="F5" s="83" t="n"/>
+      <c r="G5" s="51" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="H5" s="52" t="inlineStr">
+      <c r="H5" s="51" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="I5" s="79" t="n"/>
-      <c r="J5" s="50" t="inlineStr">
+      <c r="I5" s="83" t="n"/>
+      <c r="J5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="K5" s="50" t="inlineStr">
+      <c r="K5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="L5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="M5" s="50" t="inlineStr">
+      <c r="M5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="N5" s="50" t="inlineStr">
+      <c r="N5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="O5" s="50" t="inlineStr">
+      <c r="O5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="P5" s="50" t="inlineStr">
+      <c r="P5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q5" s="50" t="inlineStr">
+      <c r="Q5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="R5" s="79" t="n"/>
-      <c r="S5" s="79" t="n"/>
-      <c r="T5" s="50" t="inlineStr">
+      <c r="R5" s="83" t="n"/>
+      <c r="S5" s="83" t="n"/>
+      <c r="T5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="U5" s="50" t="inlineStr">
+      <c r="U5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="V5" s="50" t="inlineStr">
+      <c r="V5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="W5" s="50" t="inlineStr">
+      <c r="W5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="X5" s="50" t="inlineStr">
+      <c r="X5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="Y5" s="50" t="inlineStr">
+      <c r="Y5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="Z5" s="50" t="inlineStr">
+      <c r="Z5" s="49" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="AA5" s="57" t="inlineStr">
+      <c r="AA5" s="56" t="inlineStr">
         <is>
           <t>Down</t>
         </is>
@@ -9472,7 +9480,7 @@
       <c r="M6" s="12" t="inlineStr"/>
       <c r="N6" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O6" s="12" t="inlineStr"/>
@@ -9480,13 +9488,13 @@
       <c r="Q6" s="12" t="inlineStr"/>
       <c r="R6" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 1II, A1, 3I, 7</t>
+          <t>B1, 1I, 1II, A1, 3I, 7</t>
         </is>
       </c>
       <c r="S6" s="12" t="inlineStr"/>
       <c r="T6" s="11" t="inlineStr">
         <is>
-          <t>3II/5, 11/13</t>
+          <t>3II/5, 11/15</t>
         </is>
       </c>
       <c r="U6" s="12" t="inlineStr">
@@ -9547,7 +9555,7 @@
       <c r="M7" s="12" t="inlineStr"/>
       <c r="N7" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O7" s="12" t="inlineStr"/>
@@ -9557,7 +9565,7 @@
       <c r="S7" s="12" t="inlineStr"/>
       <c r="T7" s="11" t="inlineStr">
         <is>
-          <t>3II/5, 11/13</t>
+          <t>3II/5, 11/15</t>
         </is>
       </c>
       <c r="U7" s="12" t="inlineStr">
@@ -9615,7 +9623,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>11, 13</t>
+          <t>11, 15</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr"/>
@@ -9634,7 +9642,7 @@
       <c r="Q8" s="12" t="inlineStr"/>
       <c r="R8" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 3II/5, 11/13</t>
+          <t>B1, 1I, 3II/5, 11/15</t>
         </is>
       </c>
       <c r="S8" s="12" t="inlineStr"/>
@@ -9689,7 +9697,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>3I, 7, 13</t>
+          <t>3I, 7, 15</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -9709,7 +9717,7 @@
       <c r="Q9" s="12" t="inlineStr"/>
       <c r="R9" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 1II, A1, 3I, 7, 11/13</t>
+          <t>B1, 1I, 1II, A1, 3I, 7, 11/15</t>
         </is>
       </c>
       <c r="S9" s="12" t="inlineStr"/>
@@ -9773,7 +9781,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>11, 13</t>
+          <t>11, 15</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr"/>
@@ -9843,7 +9851,7 @@
       <c r="I11" s="10" t="inlineStr"/>
       <c r="J11" s="11" t="inlineStr">
         <is>
-          <t>3I, 7, 13</t>
+          <t>3I, 7, 15</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr">
@@ -9923,7 +9931,7 @@
       </c>
       <c r="K12" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="L12" s="11" t="inlineStr"/>
@@ -9942,7 +9950,7 @@
       <c r="Q12" s="12" t="inlineStr"/>
       <c r="R12" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 3II/5, 11/13</t>
+          <t>B1, 1I, 3II/5, 11/15</t>
         </is>
       </c>
       <c r="S12" s="12" t="inlineStr"/>
@@ -9997,7 +10005,7 @@
       <c r="I13" s="10" t="inlineStr"/>
       <c r="J13" s="11" t="inlineStr">
         <is>
-          <t>3I, 7, 11, 13</t>
+          <t>3I, 7, 11, 15</t>
         </is>
       </c>
       <c r="K13" s="12" t="inlineStr">
@@ -10017,7 +10025,7 @@
       <c r="Q13" s="12" t="inlineStr"/>
       <c r="R13" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 1II, A1, 3I, 7, 11/13</t>
+          <t>B1, 1I, 1II, A1, 3I, 7, 11/15</t>
         </is>
       </c>
       <c r="S13" s="12" t="inlineStr"/>
@@ -10081,7 +10089,7 @@
       </c>
       <c r="K14" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="L14" s="11" t="inlineStr"/>
@@ -10151,7 +10159,7 @@
       <c r="I15" s="10" t="inlineStr"/>
       <c r="J15" s="11" t="inlineStr">
         <is>
-          <t>3I, 7, 11, 13</t>
+          <t>3I, 7, 11, 15</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
@@ -10238,7 +10246,7 @@
       <c r="M16" s="12" t="inlineStr"/>
       <c r="N16" s="11" t="inlineStr">
         <is>
-          <t>1II, 13, 3I</t>
+          <t>1II, 15, 3I</t>
         </is>
       </c>
       <c r="O16" s="12" t="inlineStr"/>
@@ -10246,7 +10254,7 @@
       <c r="Q16" s="12" t="inlineStr"/>
       <c r="R16" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 3II/5, 9</t>
+          <t>B1, 1I, 3II/5, 9</t>
         </is>
       </c>
       <c r="S16" s="12" t="inlineStr"/>
@@ -10317,13 +10325,13 @@
       <c r="Q17" s="12" t="inlineStr"/>
       <c r="R17" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 1II, A1, 3I, 3II/5, 9</t>
+          <t>B1, 1I, 1II, A1, 3I, 3II/5, 9</t>
         </is>
       </c>
       <c r="S17" s="12" t="inlineStr"/>
       <c r="T17" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U17" s="12" t="inlineStr"/>
@@ -10384,7 +10392,7 @@
       <c r="M18" s="12" t="inlineStr"/>
       <c r="N18" s="11" t="inlineStr">
         <is>
-          <t>1II, 13, 3I</t>
+          <t>1II, 15, 3I</t>
         </is>
       </c>
       <c r="O18" s="12" t="inlineStr"/>
@@ -10461,7 +10469,7 @@
       <c r="S19" s="12" t="inlineStr"/>
       <c r="T19" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U19" s="12" t="inlineStr"/>
@@ -10522,7 +10530,7 @@
       <c r="M20" s="12" t="inlineStr"/>
       <c r="N20" s="11" t="inlineStr">
         <is>
-          <t>1II, 13, 3I</t>
+          <t>1II, 15, 3I</t>
         </is>
       </c>
       <c r="O20" s="12" t="inlineStr"/>
@@ -10530,7 +10538,7 @@
       <c r="Q20" s="12" t="inlineStr"/>
       <c r="R20" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 3II/5, 9</t>
+          <t>B1, 1I, 3II/5, 9</t>
         </is>
       </c>
       <c r="S20" s="12" t="inlineStr"/>
@@ -10597,13 +10605,13 @@
       <c r="Q21" s="12" t="inlineStr"/>
       <c r="R21" s="11" t="inlineStr">
         <is>
-          <t>D1, 1I, 1II, A1, 3I, 3II/5, 9</t>
+          <t>B1, 1I, 1II, A1, 3I, 3II/5, 9</t>
         </is>
       </c>
       <c r="S21" s="12" t="inlineStr"/>
       <c r="T21" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U21" s="12" t="inlineStr"/>
@@ -10664,7 +10672,7 @@
       <c r="M22" s="12" t="inlineStr"/>
       <c r="N22" s="11" t="inlineStr">
         <is>
-          <t>1II, 13, 3I</t>
+          <t>1II, 15, 3I</t>
         </is>
       </c>
       <c r="O22" s="12" t="inlineStr"/>
@@ -10737,7 +10745,7 @@
       <c r="S23" s="12" t="inlineStr"/>
       <c r="T23" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U23" s="12" t="inlineStr"/>
@@ -13175,310 +13183,310 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B1" s="63" t="n"/>
-      <c r="C1" s="63" t="n"/>
-      <c r="D1" s="63" t="n"/>
-      <c r="E1" s="63" t="n"/>
-      <c r="F1" s="63" t="n"/>
-      <c r="G1" s="63" t="n"/>
-      <c r="H1" s="63" t="n"/>
-      <c r="I1" s="64" t="n"/>
-      <c r="J1" s="55" t="inlineStr">
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="67" t="n"/>
+      <c r="G1" s="67" t="n"/>
+      <c r="H1" s="67" t="n"/>
+      <c r="I1" s="68" t="n"/>
+      <c r="J1" s="54" t="inlineStr">
         <is>
           <t>Interlocking</t>
         </is>
       </c>
-      <c r="K1" s="65" t="n"/>
-      <c r="L1" s="65" t="n"/>
-      <c r="M1" s="65" t="n"/>
-      <c r="N1" s="65" t="n"/>
-      <c r="O1" s="65" t="n"/>
-      <c r="P1" s="65" t="n"/>
-      <c r="Q1" s="65" t="n"/>
-      <c r="R1" s="65" t="n"/>
-      <c r="S1" s="65" t="n"/>
-      <c r="T1" s="65" t="n"/>
-      <c r="U1" s="65" t="n"/>
-      <c r="V1" s="65" t="n"/>
-      <c r="W1" s="65" t="n"/>
-      <c r="X1" s="65" t="n"/>
-      <c r="Y1" s="65" t="n"/>
-      <c r="Z1" s="65" t="n"/>
-      <c r="AA1" s="66" t="n"/>
+      <c r="K1" s="69" t="n"/>
+      <c r="L1" s="69" t="n"/>
+      <c r="M1" s="69" t="n"/>
+      <c r="N1" s="69" t="n"/>
+      <c r="O1" s="69" t="n"/>
+      <c r="P1" s="69" t="n"/>
+      <c r="Q1" s="69" t="n"/>
+      <c r="R1" s="69" t="n"/>
+      <c r="S1" s="69" t="n"/>
+      <c r="T1" s="69" t="n"/>
+      <c r="U1" s="69" t="n"/>
+      <c r="V1" s="69" t="n"/>
+      <c r="W1" s="69" t="n"/>
+      <c r="X1" s="69" t="n"/>
+      <c r="Y1" s="69" t="n"/>
+      <c r="Z1" s="69" t="n"/>
+      <c r="AA1" s="70" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="67" t="n"/>
-      <c r="I2" s="68" t="n"/>
-      <c r="J2" s="50" t="inlineStr">
+      <c r="A2" s="71" t="n"/>
+      <c r="I2" s="72" t="n"/>
+      <c r="J2" s="49" t="inlineStr">
         <is>
           <t>Required Switches</t>
         </is>
       </c>
-      <c r="K2" s="69" t="n"/>
-      <c r="L2" s="69" t="n"/>
-      <c r="M2" s="69" t="n"/>
-      <c r="N2" s="69" t="n"/>
-      <c r="O2" s="69" t="n"/>
-      <c r="P2" s="69" t="n"/>
-      <c r="Q2" s="70" t="n"/>
-      <c r="R2" s="50" t="inlineStr">
+      <c r="K2" s="73" t="n"/>
+      <c r="L2" s="73" t="n"/>
+      <c r="M2" s="73" t="n"/>
+      <c r="N2" s="73" t="n"/>
+      <c r="O2" s="73" t="n"/>
+      <c r="P2" s="73" t="n"/>
+      <c r="Q2" s="74" t="n"/>
+      <c r="R2" s="49" t="inlineStr">
         <is>
           <t>Required Sections</t>
         </is>
       </c>
-      <c r="S2" s="69" t="n"/>
-      <c r="T2" s="69" t="n"/>
-      <c r="U2" s="69" t="n"/>
-      <c r="V2" s="69" t="n"/>
-      <c r="W2" s="69" t="n"/>
-      <c r="X2" s="69" t="n"/>
-      <c r="Y2" s="70" t="n"/>
-      <c r="Z2" s="50" t="inlineStr">
+      <c r="S2" s="73" t="n"/>
+      <c r="T2" s="73" t="n"/>
+      <c r="U2" s="73" t="n"/>
+      <c r="V2" s="73" t="n"/>
+      <c r="W2" s="73" t="n"/>
+      <c r="X2" s="73" t="n"/>
+      <c r="Y2" s="74" t="n"/>
+      <c r="Z2" s="49" t="inlineStr">
         <is>
           <t>Required Blocks</t>
         </is>
       </c>
-      <c r="AA2" s="71" t="n"/>
+      <c r="AA2" s="75" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="72" t="n"/>
-      <c r="B3" s="73" t="n"/>
-      <c r="C3" s="73" t="n"/>
-      <c r="D3" s="73" t="n"/>
-      <c r="E3" s="73" t="n"/>
-      <c r="F3" s="73" t="n"/>
-      <c r="G3" s="73" t="n"/>
-      <c r="H3" s="73" t="n"/>
-      <c r="I3" s="74" t="n"/>
-      <c r="J3" s="50" t="inlineStr">
+      <c r="A3" s="76" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="78" t="n"/>
+      <c r="J3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="K3" s="71" t="n"/>
-      <c r="L3" s="50" t="inlineStr">
+      <c r="K3" s="75" t="n"/>
+      <c r="L3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="M3" s="71" t="n"/>
-      <c r="N3" s="50" t="inlineStr">
+      <c r="M3" s="75" t="n"/>
+      <c r="N3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="O3" s="69" t="n"/>
-      <c r="P3" s="69" t="n"/>
-      <c r="Q3" s="70" t="n"/>
-      <c r="R3" s="50" t="inlineStr">
+      <c r="O3" s="73" t="n"/>
+      <c r="P3" s="73" t="n"/>
+      <c r="Q3" s="74" t="n"/>
+      <c r="R3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="S3" s="50" t="inlineStr">
+      <c r="S3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="T3" s="50" t="inlineStr">
+      <c r="T3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="U3" s="69" t="n"/>
-      <c r="V3" s="69" t="n"/>
-      <c r="W3" s="69" t="n"/>
-      <c r="X3" s="69" t="n"/>
-      <c r="Y3" s="70" t="n"/>
-      <c r="Z3" s="75" t="n"/>
-      <c r="AA3" s="68" t="n"/>
+      <c r="U3" s="73" t="n"/>
+      <c r="V3" s="73" t="n"/>
+      <c r="W3" s="73" t="n"/>
+      <c r="X3" s="73" t="n"/>
+      <c r="Y3" s="74" t="n"/>
+      <c r="Z3" s="79" t="n"/>
+      <c r="AA3" s="72" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="51" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="C4" s="70" t="n"/>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="C4" s="74" t="n"/>
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="E4" s="70" t="n"/>
-      <c r="F4" s="52" t="inlineStr">
+      <c r="E4" s="74" t="n"/>
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="G4" s="52" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="H4" s="70" t="n"/>
-      <c r="I4" s="52" t="inlineStr">
+      <c r="H4" s="74" t="n"/>
+      <c r="I4" s="51" t="inlineStr">
         <is>
           <t>Obs.</t>
         </is>
       </c>
-      <c r="J4" s="76" t="n"/>
-      <c r="K4" s="74" t="n"/>
-      <c r="L4" s="76" t="n"/>
-      <c r="M4" s="74" t="n"/>
-      <c r="N4" s="50" t="inlineStr">
+      <c r="J4" s="80" t="n"/>
+      <c r="K4" s="78" t="n"/>
+      <c r="L4" s="80" t="n"/>
+      <c r="M4" s="78" t="n"/>
+      <c r="N4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="O4" s="70" t="n"/>
-      <c r="P4" s="50" t="inlineStr">
+      <c r="O4" s="74" t="n"/>
+      <c r="P4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="Q4" s="70" t="n"/>
-      <c r="R4" s="77" t="n"/>
-      <c r="S4" s="77" t="n"/>
-      <c r="T4" s="50" t="inlineStr">
+      <c r="Q4" s="74" t="n"/>
+      <c r="R4" s="81" t="n"/>
+      <c r="S4" s="81" t="n"/>
+      <c r="T4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="U4" s="69" t="n"/>
-      <c r="V4" s="70" t="n"/>
-      <c r="W4" s="50" t="inlineStr">
+      <c r="U4" s="73" t="n"/>
+      <c r="V4" s="74" t="n"/>
+      <c r="W4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="X4" s="69" t="n"/>
-      <c r="Y4" s="70" t="n"/>
-      <c r="Z4" s="76" t="n"/>
-      <c r="AA4" s="74" t="n"/>
+      <c r="X4" s="73" t="n"/>
+      <c r="Y4" s="74" t="n"/>
+      <c r="Z4" s="80" t="n"/>
+      <c r="AA4" s="78" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="78" t="n"/>
-      <c r="B5" s="52" t="inlineStr">
+      <c r="A5" s="82" t="n"/>
+      <c r="B5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="C5" s="52" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D5" s="52" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="E5" s="52" t="inlineStr">
+      <c r="E5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F5" s="79" t="n"/>
-      <c r="G5" s="52" t="inlineStr">
+      <c r="F5" s="83" t="n"/>
+      <c r="G5" s="51" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="H5" s="52" t="inlineStr">
+      <c r="H5" s="51" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="I5" s="79" t="n"/>
-      <c r="J5" s="50" t="inlineStr">
+      <c r="I5" s="83" t="n"/>
+      <c r="J5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="K5" s="50" t="inlineStr">
+      <c r="K5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="L5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="M5" s="50" t="inlineStr">
+      <c r="M5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="N5" s="50" t="inlineStr">
+      <c r="N5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="O5" s="50" t="inlineStr">
+      <c r="O5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="P5" s="50" t="inlineStr">
+      <c r="P5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q5" s="50" t="inlineStr">
+      <c r="Q5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="R5" s="79" t="n"/>
-      <c r="S5" s="79" t="n"/>
-      <c r="T5" s="50" t="inlineStr">
+      <c r="R5" s="83" t="n"/>
+      <c r="S5" s="83" t="n"/>
+      <c r="T5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="U5" s="50" t="inlineStr">
+      <c r="U5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="V5" s="50" t="inlineStr">
+      <c r="V5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="W5" s="50" t="inlineStr">
+      <c r="W5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="X5" s="50" t="inlineStr">
+      <c r="X5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="Y5" s="50" t="inlineStr">
+      <c r="Y5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="Z5" s="50" t="inlineStr">
+      <c r="Z5" s="49" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="AA5" s="57" t="inlineStr">
+      <c r="AA5" s="56" t="inlineStr">
         <is>
           <t>Down</t>
         </is>
@@ -13490,7 +13498,7 @@
       </c>
       <c r="B6" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C6" s="10" t="inlineStr">
@@ -13522,7 +13530,7 @@
       </c>
       <c r="J6" s="11" t="inlineStr">
         <is>
-          <t>13, 7, 3I, 1II</t>
+          <t>15, 7, 3I, 1II</t>
         </is>
       </c>
       <c r="K6" s="12" t="inlineStr">
@@ -13546,7 +13554,7 @@
       <c r="Q6" s="12" t="inlineStr"/>
       <c r="R6" s="11" t="inlineStr">
         <is>
-          <t>11/13, 7, 3I, A1, 1II</t>
+          <t>11/15, 7, 3I, A1, 1II</t>
         </is>
       </c>
       <c r="S6" s="12" t="inlineStr"/>
@@ -13569,7 +13577,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -13601,7 +13609,7 @@
       </c>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>13, 7, 3I, 1II</t>
+          <t>15, 7, 3I, 1II</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
@@ -13676,7 +13684,7 @@
       </c>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>11, 13, 7, 3I, 1II</t>
+          <t>11, 15, 7, 3I, 1II</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr"/>
@@ -13696,7 +13704,7 @@
       <c r="Q8" s="12" t="inlineStr"/>
       <c r="R8" s="11" t="inlineStr">
         <is>
-          <t>11/13, 7, 3I, A1, 1II</t>
+          <t>11/15, 7, 3I, A1, 1II</t>
         </is>
       </c>
       <c r="S8" s="12" t="inlineStr"/>
@@ -13751,7 +13759,7 @@
       </c>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>11, 13, 7, 3I, 1II</t>
+          <t>11, 15, 7, 3I, 1II</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr"/>
@@ -13834,7 +13842,7 @@
       <c r="M10" s="12" t="inlineStr"/>
       <c r="N10" s="11" t="inlineStr">
         <is>
-          <t>13, 1I</t>
+          <t>15, 1I</t>
         </is>
       </c>
       <c r="O10" s="12" t="inlineStr"/>
@@ -13853,7 +13861,7 @@
       </c>
       <c r="U10" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V10" s="11" t="inlineStr"/>
@@ -13917,7 +13925,7 @@
       <c r="M11" s="12" t="inlineStr"/>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>13, 1I</t>
+          <t>15, 1I</t>
         </is>
       </c>
       <c r="O11" s="12" t="inlineStr"/>
@@ -13932,7 +13940,7 @@
       </c>
       <c r="U11" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V11" s="11" t="inlineStr"/>
@@ -13996,7 +14004,7 @@
       <c r="M12" s="12" t="inlineStr"/>
       <c r="N12" s="11" t="inlineStr">
         <is>
-          <t>13, 1I</t>
+          <t>15, 1I</t>
         </is>
       </c>
       <c r="O12" s="12" t="inlineStr"/>
@@ -14015,7 +14023,7 @@
       </c>
       <c r="U12" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V12" s="11" t="inlineStr"/>
@@ -14079,7 +14087,7 @@
       <c r="M13" s="12" t="inlineStr"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>13, 1I</t>
+          <t>15, 1I</t>
         </is>
       </c>
       <c r="O13" s="12" t="inlineStr"/>
@@ -14094,7 +14102,7 @@
       </c>
       <c r="U13" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V13" s="11" t="inlineStr"/>
@@ -16825,310 +16833,310 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B1" s="63" t="n"/>
-      <c r="C1" s="63" t="n"/>
-      <c r="D1" s="63" t="n"/>
-      <c r="E1" s="63" t="n"/>
-      <c r="F1" s="63" t="n"/>
-      <c r="G1" s="63" t="n"/>
-      <c r="H1" s="63" t="n"/>
-      <c r="I1" s="64" t="n"/>
-      <c r="J1" s="55" t="inlineStr">
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="67" t="n"/>
+      <c r="G1" s="67" t="n"/>
+      <c r="H1" s="67" t="n"/>
+      <c r="I1" s="68" t="n"/>
+      <c r="J1" s="54" t="inlineStr">
         <is>
           <t>Interlocking</t>
         </is>
       </c>
-      <c r="K1" s="65" t="n"/>
-      <c r="L1" s="65" t="n"/>
-      <c r="M1" s="65" t="n"/>
-      <c r="N1" s="65" t="n"/>
-      <c r="O1" s="65" t="n"/>
-      <c r="P1" s="65" t="n"/>
-      <c r="Q1" s="65" t="n"/>
-      <c r="R1" s="65" t="n"/>
-      <c r="S1" s="65" t="n"/>
-      <c r="T1" s="65" t="n"/>
-      <c r="U1" s="65" t="n"/>
-      <c r="V1" s="65" t="n"/>
-      <c r="W1" s="65" t="n"/>
-      <c r="X1" s="65" t="n"/>
-      <c r="Y1" s="65" t="n"/>
-      <c r="Z1" s="65" t="n"/>
-      <c r="AA1" s="66" t="n"/>
+      <c r="K1" s="69" t="n"/>
+      <c r="L1" s="69" t="n"/>
+      <c r="M1" s="69" t="n"/>
+      <c r="N1" s="69" t="n"/>
+      <c r="O1" s="69" t="n"/>
+      <c r="P1" s="69" t="n"/>
+      <c r="Q1" s="69" t="n"/>
+      <c r="R1" s="69" t="n"/>
+      <c r="S1" s="69" t="n"/>
+      <c r="T1" s="69" t="n"/>
+      <c r="U1" s="69" t="n"/>
+      <c r="V1" s="69" t="n"/>
+      <c r="W1" s="69" t="n"/>
+      <c r="X1" s="69" t="n"/>
+      <c r="Y1" s="69" t="n"/>
+      <c r="Z1" s="69" t="n"/>
+      <c r="AA1" s="70" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="67" t="n"/>
-      <c r="I2" s="68" t="n"/>
-      <c r="J2" s="50" t="inlineStr">
+      <c r="A2" s="71" t="n"/>
+      <c r="I2" s="72" t="n"/>
+      <c r="J2" s="49" t="inlineStr">
         <is>
           <t>Required Switches</t>
         </is>
       </c>
-      <c r="K2" s="69" t="n"/>
-      <c r="L2" s="69" t="n"/>
-      <c r="M2" s="69" t="n"/>
-      <c r="N2" s="69" t="n"/>
-      <c r="O2" s="69" t="n"/>
-      <c r="P2" s="69" t="n"/>
-      <c r="Q2" s="70" t="n"/>
-      <c r="R2" s="50" t="inlineStr">
+      <c r="K2" s="73" t="n"/>
+      <c r="L2" s="73" t="n"/>
+      <c r="M2" s="73" t="n"/>
+      <c r="N2" s="73" t="n"/>
+      <c r="O2" s="73" t="n"/>
+      <c r="P2" s="73" t="n"/>
+      <c r="Q2" s="74" t="n"/>
+      <c r="R2" s="49" t="inlineStr">
         <is>
           <t>Required Sections</t>
         </is>
       </c>
-      <c r="S2" s="69" t="n"/>
-      <c r="T2" s="69" t="n"/>
-      <c r="U2" s="69" t="n"/>
-      <c r="V2" s="69" t="n"/>
-      <c r="W2" s="69" t="n"/>
-      <c r="X2" s="69" t="n"/>
-      <c r="Y2" s="70" t="n"/>
-      <c r="Z2" s="50" t="inlineStr">
+      <c r="S2" s="73" t="n"/>
+      <c r="T2" s="73" t="n"/>
+      <c r="U2" s="73" t="n"/>
+      <c r="V2" s="73" t="n"/>
+      <c r="W2" s="73" t="n"/>
+      <c r="X2" s="73" t="n"/>
+      <c r="Y2" s="74" t="n"/>
+      <c r="Z2" s="49" t="inlineStr">
         <is>
           <t>Required Blocks</t>
         </is>
       </c>
-      <c r="AA2" s="71" t="n"/>
+      <c r="AA2" s="75" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="72" t="n"/>
-      <c r="B3" s="73" t="n"/>
-      <c r="C3" s="73" t="n"/>
-      <c r="D3" s="73" t="n"/>
-      <c r="E3" s="73" t="n"/>
-      <c r="F3" s="73" t="n"/>
-      <c r="G3" s="73" t="n"/>
-      <c r="H3" s="73" t="n"/>
-      <c r="I3" s="74" t="n"/>
-      <c r="J3" s="50" t="inlineStr">
+      <c r="A3" s="76" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="78" t="n"/>
+      <c r="J3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="K3" s="71" t="n"/>
-      <c r="L3" s="50" t="inlineStr">
+      <c r="K3" s="75" t="n"/>
+      <c r="L3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="M3" s="71" t="n"/>
-      <c r="N3" s="50" t="inlineStr">
+      <c r="M3" s="75" t="n"/>
+      <c r="N3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="O3" s="69" t="n"/>
-      <c r="P3" s="69" t="n"/>
-      <c r="Q3" s="70" t="n"/>
-      <c r="R3" s="50" t="inlineStr">
+      <c r="O3" s="73" t="n"/>
+      <c r="P3" s="73" t="n"/>
+      <c r="Q3" s="74" t="n"/>
+      <c r="R3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="S3" s="50" t="inlineStr">
+      <c r="S3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="T3" s="50" t="inlineStr">
+      <c r="T3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="U3" s="69" t="n"/>
-      <c r="V3" s="69" t="n"/>
-      <c r="W3" s="69" t="n"/>
-      <c r="X3" s="69" t="n"/>
-      <c r="Y3" s="70" t="n"/>
-      <c r="Z3" s="75" t="n"/>
-      <c r="AA3" s="68" t="n"/>
+      <c r="U3" s="73" t="n"/>
+      <c r="V3" s="73" t="n"/>
+      <c r="W3" s="73" t="n"/>
+      <c r="X3" s="73" t="n"/>
+      <c r="Y3" s="74" t="n"/>
+      <c r="Z3" s="79" t="n"/>
+      <c r="AA3" s="72" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="51" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="C4" s="70" t="n"/>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="C4" s="74" t="n"/>
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="E4" s="70" t="n"/>
-      <c r="F4" s="52" t="inlineStr">
+      <c r="E4" s="74" t="n"/>
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="G4" s="52" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="H4" s="70" t="n"/>
-      <c r="I4" s="52" t="inlineStr">
+      <c r="H4" s="74" t="n"/>
+      <c r="I4" s="51" t="inlineStr">
         <is>
           <t>Obs.</t>
         </is>
       </c>
-      <c r="J4" s="76" t="n"/>
-      <c r="K4" s="74" t="n"/>
-      <c r="L4" s="76" t="n"/>
-      <c r="M4" s="74" t="n"/>
-      <c r="N4" s="50" t="inlineStr">
+      <c r="J4" s="80" t="n"/>
+      <c r="K4" s="78" t="n"/>
+      <c r="L4" s="80" t="n"/>
+      <c r="M4" s="78" t="n"/>
+      <c r="N4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="O4" s="70" t="n"/>
-      <c r="P4" s="50" t="inlineStr">
+      <c r="O4" s="74" t="n"/>
+      <c r="P4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="Q4" s="70" t="n"/>
-      <c r="R4" s="77" t="n"/>
-      <c r="S4" s="77" t="n"/>
-      <c r="T4" s="50" t="inlineStr">
+      <c r="Q4" s="74" t="n"/>
+      <c r="R4" s="81" t="n"/>
+      <c r="S4" s="81" t="n"/>
+      <c r="T4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="U4" s="69" t="n"/>
-      <c r="V4" s="70" t="n"/>
-      <c r="W4" s="50" t="inlineStr">
+      <c r="U4" s="73" t="n"/>
+      <c r="V4" s="74" t="n"/>
+      <c r="W4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="X4" s="69" t="n"/>
-      <c r="Y4" s="70" t="n"/>
-      <c r="Z4" s="76" t="n"/>
-      <c r="AA4" s="74" t="n"/>
+      <c r="X4" s="73" t="n"/>
+      <c r="Y4" s="74" t="n"/>
+      <c r="Z4" s="80" t="n"/>
+      <c r="AA4" s="78" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="78" t="n"/>
-      <c r="B5" s="52" t="inlineStr">
+      <c r="A5" s="82" t="n"/>
+      <c r="B5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="C5" s="52" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D5" s="52" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="E5" s="52" t="inlineStr">
+      <c r="E5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F5" s="79" t="n"/>
-      <c r="G5" s="52" t="inlineStr">
+      <c r="F5" s="83" t="n"/>
+      <c r="G5" s="51" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="H5" s="52" t="inlineStr">
+      <c r="H5" s="51" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="I5" s="79" t="n"/>
-      <c r="J5" s="50" t="inlineStr">
+      <c r="I5" s="83" t="n"/>
+      <c r="J5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="K5" s="50" t="inlineStr">
+      <c r="K5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="L5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="M5" s="50" t="inlineStr">
+      <c r="M5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="N5" s="50" t="inlineStr">
+      <c r="N5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="O5" s="50" t="inlineStr">
+      <c r="O5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="P5" s="50" t="inlineStr">
+      <c r="P5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q5" s="50" t="inlineStr">
+      <c r="Q5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="R5" s="79" t="n"/>
-      <c r="S5" s="79" t="n"/>
-      <c r="T5" s="50" t="inlineStr">
+      <c r="R5" s="83" t="n"/>
+      <c r="S5" s="83" t="n"/>
+      <c r="T5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="U5" s="50" t="inlineStr">
+      <c r="U5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="V5" s="50" t="inlineStr">
+      <c r="V5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="W5" s="50" t="inlineStr">
+      <c r="W5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="X5" s="50" t="inlineStr">
+      <c r="X5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="Y5" s="50" t="inlineStr">
+      <c r="Y5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="Z5" s="50" t="inlineStr">
+      <c r="Z5" s="49" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="AA5" s="57" t="inlineStr">
+      <c r="AA5" s="56" t="inlineStr">
         <is>
           <t>Down</t>
         </is>
@@ -17145,7 +17153,7 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -17207,7 +17215,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C7" s="10" t="inlineStr">
@@ -17239,7 +17247,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>13, 7, 3I</t>
+          <t>15, 7, 3I</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
@@ -17286,7 +17294,7 @@
       </c>
       <c r="B8" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C8" s="10" t="inlineStr">
@@ -17318,7 +17326,7 @@
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="11" t="inlineStr">
         <is>
-          <t>13, 7, 3I</t>
+          <t>15, 7, 3I</t>
         </is>
       </c>
       <c r="K8" s="12" t="inlineStr">
@@ -17393,7 +17401,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>11, 13, 7, 3I</t>
+          <t>11, 15, 7, 3I</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr"/>
@@ -17468,7 +17476,7 @@
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="11" t="inlineStr">
         <is>
-          <t>11, 13, 7, 3I</t>
+          <t>11, 15, 7, 3I</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr"/>
@@ -17555,7 +17563,7 @@
       <c r="M11" s="12" t="inlineStr"/>
       <c r="N11" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O11" s="12" t="inlineStr"/>
@@ -17574,7 +17582,7 @@
       </c>
       <c r="U11" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V11" s="11" t="inlineStr"/>
@@ -17638,7 +17646,7 @@
       </c>
       <c r="N12" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O12" s="12" t="inlineStr"/>
@@ -17653,7 +17661,7 @@
       </c>
       <c r="U12" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V12" s="11" t="inlineStr"/>
@@ -17713,7 +17721,7 @@
       <c r="M13" s="12" t="inlineStr"/>
       <c r="N13" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O13" s="12" t="inlineStr"/>
@@ -17732,7 +17740,7 @@
       </c>
       <c r="U13" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V13" s="11" t="inlineStr"/>
@@ -17792,7 +17800,7 @@
       </c>
       <c r="N14" s="11" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="O14" s="12" t="inlineStr"/>
@@ -17807,7 +17815,7 @@
       </c>
       <c r="U14" s="12" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="V14" s="11" t="inlineStr"/>
@@ -17876,7 +17884,7 @@
       </c>
       <c r="O15" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P15" s="11" t="inlineStr">
@@ -17955,7 +17963,7 @@
       </c>
       <c r="O16" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P16" s="11" t="inlineStr"/>
@@ -17977,7 +17985,7 @@
       </c>
       <c r="B17" s="9" t="inlineStr">
         <is>
-          <t>S2/M2</t>
+          <t>S20/M20</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
@@ -17992,7 +18000,7 @@
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="F17" s="9" t="inlineStr">
@@ -18010,7 +18018,7 @@
       </c>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>11, 13</t>
+          <t>11, 15</t>
         </is>
       </c>
       <c r="L17" s="11" t="inlineStr"/>
@@ -18063,7 +18071,7 @@
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="F18" s="9" t="inlineStr">
@@ -18081,7 +18089,7 @@
       </c>
       <c r="K18" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="L18" s="11" t="inlineStr"/>
@@ -18134,7 +18142,7 @@
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="F19" s="9" t="inlineStr">
@@ -18159,7 +18167,7 @@
       <c r="M19" s="12" t="inlineStr"/>
       <c r="N19" s="11" t="inlineStr">
         <is>
-          <t>13, 3I, 1II</t>
+          <t>15, 3I, 1II</t>
         </is>
       </c>
       <c r="O19" s="12" t="inlineStr"/>
@@ -18197,7 +18205,7 @@
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -18222,7 +18230,7 @@
       <c r="M20" s="12" t="inlineStr"/>
       <c r="N20" s="11" t="inlineStr">
         <is>
-          <t>13, 3I, 1II</t>
+          <t>15, 3I, 1II</t>
         </is>
       </c>
       <c r="O20" s="12" t="inlineStr"/>
@@ -18260,7 +18268,7 @@
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="F21" s="9" t="inlineStr">
@@ -20783,310 +20791,310 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="53" t="inlineStr">
+      <c r="A1" s="52" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="B1" s="63" t="n"/>
-      <c r="C1" s="63" t="n"/>
-      <c r="D1" s="63" t="n"/>
-      <c r="E1" s="63" t="n"/>
-      <c r="F1" s="63" t="n"/>
-      <c r="G1" s="63" t="n"/>
-      <c r="H1" s="63" t="n"/>
-      <c r="I1" s="64" t="n"/>
-      <c r="J1" s="55" t="inlineStr">
+      <c r="B1" s="67" t="n"/>
+      <c r="C1" s="67" t="n"/>
+      <c r="D1" s="67" t="n"/>
+      <c r="E1" s="67" t="n"/>
+      <c r="F1" s="67" t="n"/>
+      <c r="G1" s="67" t="n"/>
+      <c r="H1" s="67" t="n"/>
+      <c r="I1" s="68" t="n"/>
+      <c r="J1" s="54" t="inlineStr">
         <is>
           <t>Interlocking</t>
         </is>
       </c>
-      <c r="K1" s="65" t="n"/>
-      <c r="L1" s="65" t="n"/>
-      <c r="M1" s="65" t="n"/>
-      <c r="N1" s="65" t="n"/>
-      <c r="O1" s="65" t="n"/>
-      <c r="P1" s="65" t="n"/>
-      <c r="Q1" s="65" t="n"/>
-      <c r="R1" s="65" t="n"/>
-      <c r="S1" s="65" t="n"/>
-      <c r="T1" s="65" t="n"/>
-      <c r="U1" s="65" t="n"/>
-      <c r="V1" s="65" t="n"/>
-      <c r="W1" s="65" t="n"/>
-      <c r="X1" s="65" t="n"/>
-      <c r="Y1" s="65" t="n"/>
-      <c r="Z1" s="65" t="n"/>
-      <c r="AA1" s="66" t="n"/>
+      <c r="K1" s="69" t="n"/>
+      <c r="L1" s="69" t="n"/>
+      <c r="M1" s="69" t="n"/>
+      <c r="N1" s="69" t="n"/>
+      <c r="O1" s="69" t="n"/>
+      <c r="P1" s="69" t="n"/>
+      <c r="Q1" s="69" t="n"/>
+      <c r="R1" s="69" t="n"/>
+      <c r="S1" s="69" t="n"/>
+      <c r="T1" s="69" t="n"/>
+      <c r="U1" s="69" t="n"/>
+      <c r="V1" s="69" t="n"/>
+      <c r="W1" s="69" t="n"/>
+      <c r="X1" s="69" t="n"/>
+      <c r="Y1" s="69" t="n"/>
+      <c r="Z1" s="69" t="n"/>
+      <c r="AA1" s="70" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="67" t="n"/>
-      <c r="I2" s="68" t="n"/>
-      <c r="J2" s="50" t="inlineStr">
+      <c r="A2" s="71" t="n"/>
+      <c r="I2" s="72" t="n"/>
+      <c r="J2" s="49" t="inlineStr">
         <is>
           <t>Required Switches</t>
         </is>
       </c>
-      <c r="K2" s="69" t="n"/>
-      <c r="L2" s="69" t="n"/>
-      <c r="M2" s="69" t="n"/>
-      <c r="N2" s="69" t="n"/>
-      <c r="O2" s="69" t="n"/>
-      <c r="P2" s="69" t="n"/>
-      <c r="Q2" s="70" t="n"/>
-      <c r="R2" s="50" t="inlineStr">
+      <c r="K2" s="73" t="n"/>
+      <c r="L2" s="73" t="n"/>
+      <c r="M2" s="73" t="n"/>
+      <c r="N2" s="73" t="n"/>
+      <c r="O2" s="73" t="n"/>
+      <c r="P2" s="73" t="n"/>
+      <c r="Q2" s="74" t="n"/>
+      <c r="R2" s="49" t="inlineStr">
         <is>
           <t>Required Sections</t>
         </is>
       </c>
-      <c r="S2" s="69" t="n"/>
-      <c r="T2" s="69" t="n"/>
-      <c r="U2" s="69" t="n"/>
-      <c r="V2" s="69" t="n"/>
-      <c r="W2" s="69" t="n"/>
-      <c r="X2" s="69" t="n"/>
-      <c r="Y2" s="70" t="n"/>
-      <c r="Z2" s="50" t="inlineStr">
+      <c r="S2" s="73" t="n"/>
+      <c r="T2" s="73" t="n"/>
+      <c r="U2" s="73" t="n"/>
+      <c r="V2" s="73" t="n"/>
+      <c r="W2" s="73" t="n"/>
+      <c r="X2" s="73" t="n"/>
+      <c r="Y2" s="74" t="n"/>
+      <c r="Z2" s="49" t="inlineStr">
         <is>
           <t>Required Blocks</t>
         </is>
       </c>
-      <c r="AA2" s="71" t="n"/>
+      <c r="AA2" s="75" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="72" t="n"/>
-      <c r="B3" s="73" t="n"/>
-      <c r="C3" s="73" t="n"/>
-      <c r="D3" s="73" t="n"/>
-      <c r="E3" s="73" t="n"/>
-      <c r="F3" s="73" t="n"/>
-      <c r="G3" s="73" t="n"/>
-      <c r="H3" s="73" t="n"/>
-      <c r="I3" s="74" t="n"/>
-      <c r="J3" s="50" t="inlineStr">
+      <c r="A3" s="76" t="n"/>
+      <c r="B3" s="77" t="n"/>
+      <c r="C3" s="77" t="n"/>
+      <c r="D3" s="77" t="n"/>
+      <c r="E3" s="77" t="n"/>
+      <c r="F3" s="77" t="n"/>
+      <c r="G3" s="77" t="n"/>
+      <c r="H3" s="77" t="n"/>
+      <c r="I3" s="78" t="n"/>
+      <c r="J3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="K3" s="71" t="n"/>
-      <c r="L3" s="50" t="inlineStr">
+      <c r="K3" s="75" t="n"/>
+      <c r="L3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="M3" s="71" t="n"/>
-      <c r="N3" s="50" t="inlineStr">
+      <c r="M3" s="75" t="n"/>
+      <c r="N3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="O3" s="69" t="n"/>
-      <c r="P3" s="69" t="n"/>
-      <c r="Q3" s="70" t="n"/>
-      <c r="R3" s="50" t="inlineStr">
+      <c r="O3" s="73" t="n"/>
+      <c r="P3" s="73" t="n"/>
+      <c r="Q3" s="74" t="n"/>
+      <c r="R3" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="S3" s="50" t="inlineStr">
+      <c r="S3" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="T3" s="50" t="inlineStr">
+      <c r="T3" s="49" t="inlineStr">
         <is>
           <t>Flank Protection</t>
         </is>
       </c>
-      <c r="U3" s="69" t="n"/>
-      <c r="V3" s="69" t="n"/>
-      <c r="W3" s="69" t="n"/>
-      <c r="X3" s="69" t="n"/>
-      <c r="Y3" s="70" t="n"/>
-      <c r="Z3" s="75" t="n"/>
-      <c r="AA3" s="68" t="n"/>
+      <c r="U3" s="73" t="n"/>
+      <c r="V3" s="73" t="n"/>
+      <c r="W3" s="73" t="n"/>
+      <c r="X3" s="73" t="n"/>
+      <c r="Y3" s="74" t="n"/>
+      <c r="Z3" s="79" t="n"/>
+      <c r="AA3" s="72" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="51" t="inlineStr">
+      <c r="A4" s="50" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="B4" s="52" t="inlineStr">
+      <c r="B4" s="51" t="inlineStr">
         <is>
           <t>Origin</t>
         </is>
       </c>
-      <c r="C4" s="70" t="n"/>
-      <c r="D4" s="52" t="inlineStr">
+      <c r="C4" s="74" t="n"/>
+      <c r="D4" s="51" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="E4" s="70" t="n"/>
-      <c r="F4" s="52" t="inlineStr">
+      <c r="E4" s="74" t="n"/>
+      <c r="F4" s="51" t="inlineStr">
         <is>
           <t>Regime</t>
         </is>
       </c>
-      <c r="G4" s="52" t="inlineStr">
+      <c r="G4" s="51" t="inlineStr">
         <is>
           <t>Alternative</t>
         </is>
       </c>
-      <c r="H4" s="70" t="n"/>
-      <c r="I4" s="52" t="inlineStr">
+      <c r="H4" s="74" t="n"/>
+      <c r="I4" s="51" t="inlineStr">
         <is>
           <t>Obs.</t>
         </is>
       </c>
-      <c r="J4" s="76" t="n"/>
-      <c r="K4" s="74" t="n"/>
-      <c r="L4" s="76" t="n"/>
-      <c r="M4" s="74" t="n"/>
-      <c r="N4" s="50" t="inlineStr">
+      <c r="J4" s="80" t="n"/>
+      <c r="K4" s="78" t="n"/>
+      <c r="L4" s="80" t="n"/>
+      <c r="M4" s="78" t="n"/>
+      <c r="N4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="O4" s="70" t="n"/>
-      <c r="P4" s="50" t="inlineStr">
+      <c r="O4" s="74" t="n"/>
+      <c r="P4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="Q4" s="70" t="n"/>
-      <c r="R4" s="77" t="n"/>
-      <c r="S4" s="77" t="n"/>
-      <c r="T4" s="50" t="inlineStr">
+      <c r="Q4" s="74" t="n"/>
+      <c r="R4" s="81" t="n"/>
+      <c r="S4" s="81" t="n"/>
+      <c r="T4" s="49" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="U4" s="69" t="n"/>
-      <c r="V4" s="70" t="n"/>
-      <c r="W4" s="50" t="inlineStr">
+      <c r="U4" s="73" t="n"/>
+      <c r="V4" s="74" t="n"/>
+      <c r="W4" s="49" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="X4" s="69" t="n"/>
-      <c r="Y4" s="70" t="n"/>
-      <c r="Z4" s="76" t="n"/>
-      <c r="AA4" s="74" t="n"/>
+      <c r="X4" s="73" t="n"/>
+      <c r="Y4" s="74" t="n"/>
+      <c r="Z4" s="80" t="n"/>
+      <c r="AA4" s="78" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="78" t="n"/>
-      <c r="B5" s="52" t="inlineStr">
+      <c r="A5" s="82" t="n"/>
+      <c r="B5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="C5" s="52" t="inlineStr">
+      <c r="C5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="D5" s="52" t="inlineStr">
+      <c r="D5" s="51" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="E5" s="52" t="inlineStr">
+      <c r="E5" s="51" t="inlineStr">
         <is>
           <t>Location</t>
         </is>
       </c>
-      <c r="F5" s="79" t="n"/>
-      <c r="G5" s="52" t="inlineStr">
+      <c r="F5" s="83" t="n"/>
+      <c r="G5" s="51" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="H5" s="52" t="inlineStr">
+      <c r="H5" s="51" t="inlineStr">
         <is>
           <t>Route</t>
         </is>
       </c>
-      <c r="I5" s="79" t="n"/>
-      <c r="J5" s="50" t="inlineStr">
+      <c r="I5" s="83" t="n"/>
+      <c r="J5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="K5" s="50" t="inlineStr">
+      <c r="K5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="L5" s="50" t="inlineStr">
+      <c r="L5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="M5" s="50" t="inlineStr">
+      <c r="M5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="N5" s="50" t="inlineStr">
+      <c r="N5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="O5" s="50" t="inlineStr">
+      <c r="O5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="P5" s="50" t="inlineStr">
+      <c r="P5" s="49" t="inlineStr">
         <is>
           <t>Normal</t>
         </is>
       </c>
-      <c r="Q5" s="50" t="inlineStr">
+      <c r="Q5" s="49" t="inlineStr">
         <is>
           <t>Reverse</t>
         </is>
       </c>
-      <c r="R5" s="79" t="n"/>
-      <c r="S5" s="79" t="n"/>
-      <c r="T5" s="50" t="inlineStr">
+      <c r="R5" s="83" t="n"/>
+      <c r="S5" s="83" t="n"/>
+      <c r="T5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="U5" s="50" t="inlineStr">
+      <c r="U5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="V5" s="50" t="inlineStr">
+      <c r="V5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="W5" s="50" t="inlineStr">
+      <c r="W5" s="49" t="inlineStr">
         <is>
           <t>Vital</t>
         </is>
       </c>
-      <c r="X5" s="50" t="inlineStr">
+      <c r="X5" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve"> Sub Vital</t>
         </is>
       </c>
-      <c r="Y5" s="50" t="inlineStr">
+      <c r="Y5" s="49" t="inlineStr">
         <is>
           <t>Remote</t>
         </is>
       </c>
-      <c r="Z5" s="50" t="inlineStr">
+      <c r="Z5" s="49" t="inlineStr">
         <is>
           <t>Up</t>
         </is>
       </c>
-      <c r="AA5" s="57" t="inlineStr">
+      <c r="AA5" s="56" t="inlineStr">
         <is>
           <t>Down</t>
         </is>
@@ -21143,7 +21151,7 @@
       </c>
       <c r="O6" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P6" s="11" t="inlineStr"/>
@@ -21193,7 +21201,7 @@
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="11" t="inlineStr">
         <is>
-          <t>3I, 7, 13</t>
+          <t>3I, 7, 15</t>
         </is>
       </c>
       <c r="K7" s="12" t="inlineStr">
@@ -21265,7 +21273,7 @@
       </c>
       <c r="K8" s="12" t="inlineStr">
         <is>
-          <t>11, 13</t>
+          <t>11, 15</t>
         </is>
       </c>
       <c r="L8" s="11" t="inlineStr"/>
@@ -21331,7 +21339,7 @@
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="11" t="inlineStr">
         <is>
-          <t>3I, 7, 11, 13</t>
+          <t>3I, 7, 11, 15</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr"/>
@@ -21399,7 +21407,7 @@
       </c>
       <c r="K10" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="L10" s="11" t="inlineStr"/>
@@ -21478,7 +21486,7 @@
       <c r="N11" s="11" t="inlineStr"/>
       <c r="O11" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P11" s="11" t="inlineStr"/>
@@ -21487,7 +21495,7 @@
       <c r="S11" s="12" t="inlineStr"/>
       <c r="T11" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U11" s="12" t="inlineStr"/>
@@ -21544,7 +21552,7 @@
       <c r="M12" s="12" t="inlineStr"/>
       <c r="N12" s="11" t="inlineStr">
         <is>
-          <t>13, 3I</t>
+          <t>15, 3I</t>
         </is>
       </c>
       <c r="O12" s="12" t="inlineStr"/>
@@ -21604,7 +21612,7 @@
       <c r="N13" s="11" t="inlineStr"/>
       <c r="O13" s="12" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>15</t>
         </is>
       </c>
       <c r="P13" s="11" t="inlineStr"/>
@@ -21613,7 +21621,7 @@
       <c r="S13" s="12" t="inlineStr"/>
       <c r="T13" s="11" t="inlineStr">
         <is>
-          <t>7, 11/13</t>
+          <t>7, 11/15</t>
         </is>
       </c>
       <c r="U13" s="12" t="inlineStr"/>
@@ -21670,7 +21678,7 @@
       <c r="M14" s="12" t="inlineStr"/>
       <c r="N14" s="11" t="inlineStr">
         <is>
-          <t>13, 3I</t>
+          <t>15, 3I</t>
         </is>
       </c>
       <c r="O14" s="12" t="inlineStr"/>
@@ -21698,7 +21706,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="D15" s="9" t="inlineStr">
@@ -24398,24 +24406,24 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="58" t="inlineStr">
+      <c r="A1" s="57" t="inlineStr">
         <is>
           <t>Overlap</t>
         </is>
       </c>
-      <c r="B1" s="66" t="n"/>
-      <c r="C1" s="55" t="inlineStr">
+      <c r="B1" s="70" t="n"/>
+      <c r="C1" s="54" t="inlineStr">
         <is>
           <t>Approach Route Cancel</t>
         </is>
       </c>
-      <c r="D1" s="66" t="n"/>
-      <c r="E1" s="55" t="inlineStr">
+      <c r="D1" s="70" t="n"/>
+      <c r="E1" s="54" t="inlineStr">
         <is>
           <t>Emergency Route Cancel</t>
         </is>
       </c>
-      <c r="F1" s="66" t="n"/>
+      <c r="F1" s="70" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -24423,27 +24431,27 @@
           <t>Track</t>
         </is>
       </c>
-      <c r="B2" s="50" t="inlineStr">
+      <c r="B2" s="49" t="inlineStr">
         <is>
           <t>Delay [s]</t>
         </is>
       </c>
-      <c r="C2" s="50" t="inlineStr">
+      <c r="C2" s="49" t="inlineStr">
         <is>
           <t>Signal</t>
         </is>
       </c>
-      <c r="D2" s="50" t="inlineStr">
+      <c r="D2" s="49" t="inlineStr">
         <is>
           <t>Delay [s]</t>
         </is>
       </c>
-      <c r="E2" s="50" t="inlineStr">
+      <c r="E2" s="49" t="inlineStr">
         <is>
           <t>Destination</t>
         </is>
       </c>
-      <c r="F2" s="57" t="inlineStr">
+      <c r="F2" s="56" t="inlineStr">
         <is>
           <t>Delay [s]</t>
         </is>
@@ -24452,7 +24460,7 @@
     <row r="3">
       <c r="A3" s="32" t="inlineStr">
         <is>
-          <t>11/13</t>
+          <t>11/15</t>
         </is>
       </c>
       <c r="B3" s="12" t="n">
@@ -24610,7 +24618,7 @@
       <c r="D11" s="12" t="n"/>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="F11" s="13" t="n">
@@ -25022,7 +25030,7 @@
       </c>
       <c r="D2" s="40" t="inlineStr">
         <is>
-          <t xml:space="preserve">station_name Cascais
+          <t xml:space="preserve">station_name Cascais (NOT REAL DATA - FOR TESTING ONLY)
 </t>
         </is>
       </c>
@@ -25036,7 +25044,7 @@
       </c>
       <c r="B3" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    1II 24980 24908 24749
+          <t xml:space="preserve">    1II 64980 64908 64749
 </t>
         </is>
       </c>
@@ -25062,7 +25070,7 @@
       </c>
       <c r="B4" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    D1 24869 24749
+          <t xml:space="preserve">    B1 64869 64749
 </t>
         </is>
       </c>
@@ -25088,7 +25096,7 @@
       </c>
       <c r="B5" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    1I 24908 25100 24869
+          <t xml:space="preserve">    1I 64908 65100 64869
 </t>
         </is>
       </c>
@@ -25114,7 +25122,7 @@
       </c>
       <c r="B6" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    A1 25100 24980
+          <t xml:space="preserve">    A1 65100 64980
 </t>
         </is>
       </c>
@@ -25140,7 +25148,7 @@
       </c>
       <c r="B7" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3I 25174 25141 25100
+          <t xml:space="preserve">    3I 65174 65141 65100
 </t>
         </is>
       </c>
@@ -25161,7 +25169,7 @@
       </c>
       <c r="B8" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3II/5 25185 25192 25100 25141
+          <t xml:space="preserve">    3II/5 65185 65192 65100 65141
 </t>
         </is>
       </c>
@@ -25182,7 +25190,7 @@
       </c>
       <c r="B9" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    7 25230 25210 25174
+          <t xml:space="preserve">    7 65230 65210 65174
 </t>
         </is>
       </c>
@@ -25203,7 +25211,7 @@
       </c>
       <c r="B10" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    11/13 25280 25280 25185 25210
+          <t xml:space="preserve">    11/15 65280 65280 65185 65210
 </t>
         </is>
       </c>
@@ -25224,7 +25232,7 @@
       </c>
       <c r="B11" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    9 25258 25258 25192
+          <t xml:space="preserve">    9 65258 65258 65192
 </t>
         </is>
       </c>
@@ -25239,13 +25247,13 @@
     <row r="12">
       <c r="A12" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEC D1
+          <t xml:space="preserve">SEC B1
 </t>
         </is>
       </c>
       <c r="B12" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    R1 25410 25230
+          <t xml:space="preserve">    R1 65410 65230
 </t>
         </is>
       </c>
@@ -25266,7 +25274,7 @@
       </c>
       <c r="B13" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    I 25423 25280
+          <t xml:space="preserve">    I 65423 65280
 </t>
         </is>
       </c>
@@ -25287,7 +25295,7 @@
       </c>
       <c r="B14" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    II 25423 25280
+          <t xml:space="preserve">    II 65423 65280
 </t>
         </is>
       </c>
@@ -25308,7 +25316,7 @@
       </c>
       <c r="B15" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    III 25423 25258
+          <t xml:space="preserve">    III 65423 65258
 </t>
         </is>
       </c>
@@ -25329,7 +25337,7 @@
       </c>
       <c r="B16" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    IV 25423 25258
+          <t xml:space="preserve">    IV 65423 65258
 </t>
         </is>
       </c>
@@ -25370,7 +25378,7 @@
       </c>
       <c r="B18" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    1I 24889 24960
+          <t xml:space="preserve">    1I 64889 64960
 </t>
         </is>
       </c>
@@ -25390,7 +25398,7 @@
       </c>
       <c r="B19" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    1II 24960 24889
+          <t xml:space="preserve">    1II 64960 64889
 </t>
         </is>
       </c>
@@ -25404,13 +25412,13 @@
     <row r="20">
       <c r="A20" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NDE C D1
+          <t xml:space="preserve">    NDE C B1
 </t>
         </is>
       </c>
       <c r="B20" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3I 25120 25168
+          <t xml:space="preserve">    3I 65120 65168
 </t>
         </is>
       </c>
@@ -25430,7 +25438,7 @@
       </c>
       <c r="B21" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3II 25180 25120
+          <t xml:space="preserve">    3II 65180 65120
 </t>
         </is>
       </c>
@@ -25450,7 +25458,7 @@
       </c>
       <c r="B22" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    5 25157 25199
+          <t xml:space="preserve">    5 65157 65199
 </t>
         </is>
       </c>
@@ -25470,7 +25478,7 @@
       </c>
       <c r="B23" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    7 25181 25224
+          <t xml:space="preserve">    7 65181 65224
 </t>
         </is>
       </c>
@@ -25490,7 +25498,7 @@
       </c>
       <c r="B24" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    9 25194 25252
+          <t xml:space="preserve">    9 65194 65252
 </t>
         </is>
       </c>
@@ -25510,7 +25518,7 @@
       </c>
       <c r="B25" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    11 25217 25274
+          <t xml:space="preserve">    11 65217 65274
 </t>
         </is>
       </c>
@@ -25530,7 +25538,7 @@
       </c>
       <c r="B26" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    13 25256 25191
+          <t xml:space="preserve">    15 65256 65191
 </t>
         </is>
       </c>
@@ -25570,7 +25578,7 @@
       </c>
       <c r="B28" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    S1 24741 23791 350
+          <t xml:space="preserve">    S1 64741 63791 350
 </t>
         </is>
       </c>
@@ -25590,7 +25598,7 @@
       </c>
       <c r="B29" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    SC1 24741 23794 350
+          <t xml:space="preserve">    SC1 64741 63794 350
 </t>
         </is>
       </c>
@@ -25610,7 +25618,7 @@
       </c>
       <c r="B30" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    M_SPE2 24774
+          <t xml:space="preserve">    M_SPE2 64774
 </t>
         </is>
       </c>
@@ -25625,7 +25633,7 @@
       </c>
       <c r="B31" s="39" t="inlineStr">
         <is>
-          <t xml:space="preserve">    M1 24868
+          <t xml:space="preserve">    M1 64868
 </t>
         </is>
       </c>
@@ -25634,13 +25642,13 @@
     <row r="32">
       <c r="A32" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NDE A 11/13 -
+          <t xml:space="preserve">    NDE A 11/15 -
 </t>
         </is>
       </c>
       <c r="B32" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    M12 24981
+          <t xml:space="preserve">    M12 64981
 </t>
         </is>
       </c>
@@ -25654,7 +25662,7 @@
       </c>
       <c r="B33" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    M3 25099
+          <t xml:space="preserve">    M3 65099
 </t>
         </is>
       </c>
@@ -25668,7 +25676,7 @@
       </c>
       <c r="B34" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    M5 25099
+          <t xml:space="preserve">    M5 65099
 </t>
         </is>
       </c>
@@ -25682,7 +25690,7 @@
       </c>
       <c r="B35" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    M10 25231
+          <t xml:space="preserve">    M10 65231
 </t>
         </is>
       </c>
@@ -25696,7 +25704,7 @@
       </c>
       <c r="B36" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    S2/M2 25275
+          <t xml:space="preserve">    S20/M20 65275
 </t>
         </is>
       </c>
@@ -25710,7 +25718,7 @@
       </c>
       <c r="B37" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    S4/M4 25275
+          <t xml:space="preserve">    S4/M4 65275
 </t>
         </is>
       </c>
@@ -25724,7 +25732,7 @@
       </c>
       <c r="B38" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    S6/M6 25263
+          <t xml:space="preserve">    S6/M6 65263
 </t>
         </is>
       </c>
@@ -25738,7 +25746,7 @@
       </c>
       <c r="B39" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    S8/M8 25263
+          <t xml:space="preserve">    S8/M8 65263
 </t>
         </is>
       </c>
@@ -25773,7 +25781,7 @@
     <row r="43">
       <c r="A43" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NDE B 11/13
+          <t xml:space="preserve">    NDE B 11/15
 </t>
         </is>
       </c>
@@ -25791,7 +25799,7 @@
     <row r="45">
       <c r="A45" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">SEC 11/13 TJD
+          <t xml:space="preserve">SEC 11/15 TJD
 </t>
         </is>
       </c>
@@ -25809,7 +25817,7 @@
     <row r="47">
       <c r="A47" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">        SWP S2/M2
+          <t xml:space="preserve">        SWP S20/M20
 </t>
         </is>
       </c>
@@ -25854,7 +25862,7 @@
     <row r="52">
       <c r="A52" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">        SWI 13
+          <t xml:space="preserve">        SWI 15
 </t>
         </is>
       </c>
@@ -25980,7 +25988,7 @@
     <row r="66">
       <c r="A66" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NDE B 11/13
+          <t xml:space="preserve">    NDE B 11/15
 </t>
         </is>
       </c>
@@ -26007,7 +26015,7 @@
     <row r="69">
       <c r="A69" s="38" t="inlineStr">
         <is>
-          <t xml:space="preserve">    NDE B 11/13
+          <t xml:space="preserve">    NDE B 11/15
 </t>
         </is>
       </c>

</xml_diff>